<commit_message>
chore: republish forecasts (neuro+Dengue) + reselect ISO (0 cambios neuro)
predict-all (General) regenero los all_forecast con AMBAS cohortes (resuelve el estado
Dengue-only). reselect con alineacion ISO: 0/333 cambios en neuro (suave + reglas robustas
al desfase de 1 sem; el bug solo afectaba a Dengue por volatilidad). Tabla 333 con columnas
de auditoria ahora ISO-correctas, modelo_produccion intacto. Dengue 54/45 (±1 ruido DeepAR).
dvc push (1733 archivos).
</commit_message>
<xml_diff>
--- a/reports/ProdDetails/produccion_dengue.xlsx
+++ b/reports/ProdDetails/produccion_dengue.xlsx
@@ -578,9 +578,11 @@
         <v>200</v>
       </c>
       <c r="K2" t="n">
-        <v>0.008980106835938563</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
+        <v>0.008620340954539604</v>
+      </c>
+      <c r="L2" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M2" t="n">
         <v>200</v>
       </c>
@@ -654,9 +656,11 @@
         <v>200</v>
       </c>
       <c r="K3" t="n">
-        <v>0.01223255052547364</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
+        <v>0.01293774852062258</v>
+      </c>
+      <c r="L3" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M3" t="n">
         <v>200</v>
       </c>
@@ -730,9 +734,11 @@
         <v>200</v>
       </c>
       <c r="K4" t="n">
-        <v>0.07902433993532074</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
+        <v>0.07625688786245192</v>
+      </c>
+      <c r="L4" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M4" t="n">
         <v>200</v>
       </c>
@@ -803,12 +809,14 @@
         <v>175.1088701866436</v>
       </c>
       <c r="J5" t="n">
-        <v>199.3234195740198</v>
+        <v>199.2843630995856</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1167777980905749</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
+        <v>0.1172378734304398</v>
+      </c>
+      <c r="L5" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M5" t="n">
         <v>200</v>
       </c>
@@ -879,12 +887,14 @@
         <v>191.646475967384</v>
       </c>
       <c r="J6" t="n">
-        <v>199.9904719366027</v>
+        <v>199.9861671147559</v>
       </c>
       <c r="K6" t="n">
-        <v>0.05344732191053987</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
+        <v>0.05340157993507275</v>
+      </c>
+      <c r="L6" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M6" t="n">
         <v>200</v>
       </c>
@@ -955,12 +965,14 @@
         <v>186.9197740801393</v>
       </c>
       <c r="J7" t="n">
-        <v>199.9920711524921</v>
+        <v>199.9884309380623</v>
       </c>
       <c r="K7" t="n">
-        <v>0.05301641570428982</v>
-      </c>
-      <c r="L7" t="inlineStr"/>
+        <v>0.05308000538193182</v>
+      </c>
+      <c r="L7" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M7" t="n">
         <v>200</v>
       </c>
@@ -1031,12 +1043,14 @@
         <v>154.5040916050135</v>
       </c>
       <c r="J8" t="n">
-        <v>49.448315629151</v>
+        <v>48.2035225269852</v>
       </c>
       <c r="K8" t="n">
-        <v>3.415782015598385</v>
-      </c>
-      <c r="L8" t="inlineStr"/>
+        <v>3.314891306805234</v>
+      </c>
+      <c r="L8" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M8" t="n">
         <v>95.80329746013628</v>
       </c>
@@ -1066,11 +1080,11 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>49.448315629151</v>
+        <v>48.2035225269852</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=49.45% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=48.20% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1123,14 @@
         <v>164.086229256472</v>
       </c>
       <c r="J9" t="n">
-        <v>76.1592104766909</v>
+        <v>69.98966250353146</v>
       </c>
       <c r="K9" t="n">
-        <v>3.688325335653582</v>
-      </c>
-      <c r="L9" t="inlineStr"/>
+        <v>2.063113567141357</v>
+      </c>
+      <c r="L9" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M9" t="n">
         <v>111.3394980759131</v>
       </c>
@@ -1144,11 +1160,11 @@
         </is>
       </c>
       <c r="U9" t="n">
-        <v>76.1592104766909</v>
+        <v>69.98966250353146</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=76.16% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=69.99% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1187,12 +1203,14 @@
         <v>164.4874496413386</v>
       </c>
       <c r="J10" t="n">
-        <v>42.29469737291846</v>
+        <v>45.23277359273659</v>
       </c>
       <c r="K10" t="n">
-        <v>1.605336268698746</v>
-      </c>
-      <c r="L10" t="inlineStr"/>
+        <v>1.634276789548177</v>
+      </c>
+      <c r="L10" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M10" t="n">
         <v>95.95074714452349</v>
       </c>
@@ -1222,11 +1240,11 @@
         </is>
       </c>
       <c r="U10" t="n">
-        <v>42.29469737291846</v>
+        <v>45.23277359273659</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=42.29% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=45.23% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1265,12 +1283,14 @@
         <v>123.2554563734294</v>
       </c>
       <c r="J11" t="n">
-        <v>198.0872324051026</v>
+        <v>198.0164154965292</v>
       </c>
       <c r="K11" t="n">
-        <v>0.5883275269435004</v>
-      </c>
-      <c r="L11" t="inlineStr"/>
+        <v>0.5887372433414818</v>
+      </c>
+      <c r="L11" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M11" t="n">
         <v>192.4219018577286</v>
       </c>
@@ -1343,12 +1363,14 @@
         <v>147.3485671696691</v>
       </c>
       <c r="J12" t="n">
-        <v>199.5587784261111</v>
+        <v>199.523179310629</v>
       </c>
       <c r="K12" t="n">
-        <v>0.3711322500993692</v>
-      </c>
-      <c r="L12" t="inlineStr"/>
+        <v>0.3712791089096222</v>
+      </c>
+      <c r="L12" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M12" t="n">
         <v>191.5362391585139</v>
       </c>
@@ -1419,12 +1441,14 @@
         <v>157.1522264328246</v>
       </c>
       <c r="J13" t="n">
-        <v>199.8393822352099</v>
+        <v>199.8262982460481</v>
       </c>
       <c r="K13" t="n">
-        <v>0.2121195042665527</v>
-      </c>
-      <c r="L13" t="inlineStr"/>
+        <v>0.2119254300762861</v>
+      </c>
+      <c r="L13" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M13" t="n">
         <v>194.1951423424674</v>
       </c>
@@ -1495,12 +1519,14 @@
         <v>66.61025297793201</v>
       </c>
       <c r="J14" t="n">
-        <v>84.9403327767854</v>
+        <v>85.47396170872173</v>
       </c>
       <c r="K14" t="n">
-        <v>2.624469817249901</v>
-      </c>
-      <c r="L14" t="inlineStr"/>
+        <v>2.660604966823898</v>
+      </c>
+      <c r="L14" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M14" t="n">
         <v>168.2605793498451</v>
       </c>
@@ -1573,12 +1599,14 @@
         <v>82.6747998505866</v>
       </c>
       <c r="J15" t="n">
-        <v>90.82996398527685</v>
+        <v>89.8785759618037</v>
       </c>
       <c r="K15" t="n">
-        <v>1.202745696995517</v>
-      </c>
-      <c r="L15" t="inlineStr"/>
+        <v>1.189208099884046</v>
+      </c>
+      <c r="L15" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M15" t="n">
         <v>172.9250609621144</v>
       </c>
@@ -1651,12 +1679,14 @@
         <v>90.20708978859948</v>
       </c>
       <c r="J16" t="n">
-        <v>142.1698014999685</v>
+        <v>142.02923967689</v>
       </c>
       <c r="K16" t="n">
-        <v>1.461545414911759</v>
-      </c>
-      <c r="L16" t="inlineStr"/>
+        <v>1.457101397264992</v>
+      </c>
+      <c r="L16" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M16" t="n">
         <v>177.5562163584148</v>
       </c>
@@ -1729,12 +1759,14 @@
         <v>194.5446671655584</v>
       </c>
       <c r="J17" t="n">
-        <v>199.9347630529597</v>
+        <v>199.943152462609</v>
       </c>
       <c r="K17" t="n">
-        <v>0.05500281057855451</v>
-      </c>
-      <c r="L17" t="inlineStr"/>
+        <v>0.0548479375829464</v>
+      </c>
+      <c r="L17" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M17" t="n">
         <v>200</v>
       </c>
@@ -1808,9 +1840,11 @@
         <v>200</v>
       </c>
       <c r="K18" t="n">
-        <v>0.000582446063573821</v>
-      </c>
-      <c r="L18" t="inlineStr"/>
+        <v>0.0005657554175379</v>
+      </c>
+      <c r="L18" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
         <v>0</v>
@@ -1877,12 +1911,14 @@
         <v>196.278530387405</v>
       </c>
       <c r="J19" t="n">
-        <v>199.9010828640821</v>
+        <v>199.8695191024682</v>
       </c>
       <c r="K19" t="n">
-        <v>0.05750655344769912</v>
-      </c>
-      <c r="L19" t="inlineStr"/>
+        <v>0.05725188032739883</v>
+      </c>
+      <c r="L19" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M19" t="n">
         <v>200</v>
       </c>
@@ -1956,9 +1992,11 @@
         <v>200</v>
       </c>
       <c r="K20" t="n">
-        <v>0.001262668041030563</v>
-      </c>
-      <c r="L20" t="inlineStr"/>
+        <v>0.001370789179767052</v>
+      </c>
+      <c r="L20" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
         <v>0</v>
@@ -2028,9 +2066,11 @@
         <v>200</v>
       </c>
       <c r="K21" t="n">
-        <v>0.006155900490740383</v>
-      </c>
-      <c r="L21" t="inlineStr"/>
+        <v>0.005994552645078885</v>
+      </c>
+      <c r="L21" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
         <v>0</v>
@@ -2100,9 +2140,11 @@
         <v>200</v>
       </c>
       <c r="K22" t="n">
-        <v>0.0004386668824289527</v>
-      </c>
-      <c r="L22" t="inlineStr"/>
+        <v>0.000365936301039679</v>
+      </c>
+      <c r="L22" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
         <v>0</v>
@@ -2169,12 +2211,14 @@
         <v>149.2565324185079</v>
       </c>
       <c r="J23" t="n">
-        <v>199.2048177791976</v>
+        <v>199.2619412956352</v>
       </c>
       <c r="K23" t="n">
-        <v>0.118578293258006</v>
-      </c>
-      <c r="L23" t="inlineStr"/>
+        <v>0.1191078773049664</v>
+      </c>
+      <c r="L23" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M23" t="n">
         <v>192.8571428571429</v>
       </c>
@@ -2245,12 +2289,14 @@
         <v>156.2502876793226</v>
       </c>
       <c r="J24" t="n">
-        <v>198.7364217540033</v>
+        <v>198.5231057940479</v>
       </c>
       <c r="K24" t="n">
-        <v>0.07131395163685894</v>
-      </c>
-      <c r="L24" t="inlineStr"/>
+        <v>0.0644576519532402</v>
+      </c>
+      <c r="L24" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M24" t="n">
         <v>138.2549574812263</v>
       </c>
@@ -2271,7 +2317,7 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>DeepAR</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
@@ -2282,7 +2328,7 @@
       <c r="U24" t="inlineStr"/>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Prophet: serie casi-cero (total 1 casos), menor MAE real</t>
+          <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -2321,12 +2367,14 @@
         <v>155.3955473497874</v>
       </c>
       <c r="J25" t="n">
-        <v>199.9219951890681</v>
+        <v>199.9139299449369</v>
       </c>
       <c r="K25" t="n">
-        <v>0.05804041841012747</v>
-      </c>
-      <c r="L25" t="inlineStr"/>
+        <v>0.0576600837228529</v>
+      </c>
+      <c r="L25" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M25" t="n">
         <v>200</v>
       </c>
@@ -2400,9 +2448,11 @@
         <v>200</v>
       </c>
       <c r="K26" t="n">
-        <v>0.09487158631641658</v>
-      </c>
-      <c r="L26" t="inlineStr"/>
+        <v>0.09259454194778965</v>
+      </c>
+      <c r="L26" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M26" t="n">
         <v>200</v>
       </c>
@@ -2476,9 +2526,11 @@
         <v>200</v>
       </c>
       <c r="K27" t="n">
-        <v>0.01217744203193361</v>
-      </c>
-      <c r="L27" t="inlineStr"/>
+        <v>0.01173072176237696</v>
+      </c>
+      <c r="L27" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M27" t="n">
         <v>200</v>
       </c>
@@ -2552,9 +2604,11 @@
         <v>200</v>
       </c>
       <c r="K28" t="n">
-        <v>0.004357350598142374</v>
-      </c>
-      <c r="L28" t="inlineStr"/>
+        <v>0.004403138451811863</v>
+      </c>
+      <c r="L28" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M28" t="n">
         <v>200</v>
       </c>
@@ -2628,9 +2682,11 @@
         <v>200</v>
       </c>
       <c r="K29" t="n">
-        <v>0.02400026013487088</v>
-      </c>
-      <c r="L29" t="inlineStr"/>
+        <v>0.02627149302176331</v>
+      </c>
+      <c r="L29" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M29" t="n">
         <v>200</v>
       </c>
@@ -2704,9 +2760,11 @@
         <v>200</v>
       </c>
       <c r="K30" t="n">
-        <v>0.005648859496855605</v>
-      </c>
-      <c r="L30" t="inlineStr"/>
+        <v>0.005751018203588878</v>
+      </c>
+      <c r="L30" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M30" t="n">
         <v>200</v>
       </c>
@@ -2780,9 +2838,11 @@
         <v>200</v>
       </c>
       <c r="K31" t="n">
-        <v>0.006504246045091579</v>
-      </c>
-      <c r="L31" t="inlineStr"/>
+        <v>0.005810557376236404</v>
+      </c>
+      <c r="L31" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M31" t="n">
         <v>200</v>
       </c>
@@ -2853,12 +2913,14 @@
         <v>164.6748490827784</v>
       </c>
       <c r="J32" t="n">
-        <v>187.7116605365616</v>
+        <v>188.3994774916149</v>
       </c>
       <c r="K32" t="n">
-        <v>0.35590860162829</v>
-      </c>
-      <c r="L32" t="inlineStr"/>
+        <v>0.3600397467700314</v>
+      </c>
+      <c r="L32" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M32" t="n">
         <v>152.3809523809524</v>
       </c>
@@ -2929,12 +2991,14 @@
         <v>170.4028696730483</v>
       </c>
       <c r="J33" t="n">
-        <v>197.7160600542925</v>
+        <v>197.5602748361831</v>
       </c>
       <c r="K33" t="n">
-        <v>0.1629487095041507</v>
-      </c>
-      <c r="L33" t="inlineStr"/>
+        <v>0.3071348444317514</v>
+      </c>
+      <c r="L33" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M33" t="n">
         <v>200</v>
       </c>
@@ -3005,12 +3069,14 @@
         <v>169.6571057340244</v>
       </c>
       <c r="J34" t="n">
-        <v>172.2289143480554</v>
+        <v>171.6084043022315</v>
       </c>
       <c r="K34" t="n">
-        <v>0.4078312226593602</v>
-      </c>
-      <c r="L34" t="inlineStr"/>
+        <v>0.4006139541700345</v>
+      </c>
+      <c r="L34" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M34" t="n">
         <v>163.9888682745826</v>
       </c>
@@ -3081,12 +3147,14 @@
         <v>48.55849570822402</v>
       </c>
       <c r="J35" t="n">
-        <v>128.6317087128079</v>
+        <v>128.6246318422078</v>
       </c>
       <c r="K35" t="n">
-        <v>0.8248307660368517</v>
-      </c>
-      <c r="L35" t="inlineStr"/>
+        <v>0.8253314883004678</v>
+      </c>
+      <c r="L35" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M35" t="n">
         <v>190.1370507886782</v>
       </c>
@@ -3159,12 +3227,14 @@
         <v>58.86670393327421</v>
       </c>
       <c r="J36" t="n">
-        <v>171.3518767659004</v>
+        <v>170.6440396621451</v>
       </c>
       <c r="K36" t="n">
-        <v>0.649354005833872</v>
-      </c>
-      <c r="L36" t="inlineStr"/>
+        <v>0.6600202651972441</v>
+      </c>
+      <c r="L36" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M36" t="n">
         <v>187.6511691920828</v>
       </c>
@@ -3235,12 +3305,14 @@
         <v>60.32903496111531</v>
       </c>
       <c r="J37" t="n">
-        <v>163.1188236017408</v>
+        <v>162.0004203901676</v>
       </c>
       <c r="K37" t="n">
-        <v>0.8129319453662752</v>
-      </c>
-      <c r="L37" t="inlineStr"/>
+        <v>0.8181360894281809</v>
+      </c>
+      <c r="L37" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M37" t="n">
         <v>180.650285245381</v>
       </c>
@@ -3311,12 +3383,14 @@
         <v>164.4263244057969</v>
       </c>
       <c r="J38" t="n">
-        <v>194.5679991577052</v>
+        <v>193.5392151146532</v>
       </c>
       <c r="K38" t="n">
-        <v>0.3264860329740122</v>
-      </c>
-      <c r="L38" t="inlineStr"/>
+        <v>0.3365288969477717</v>
+      </c>
+      <c r="L38" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M38" t="n">
         <v>182.488038277512</v>
       </c>
@@ -3387,12 +3461,14 @@
         <v>170.2041702191862</v>
       </c>
       <c r="J39" t="n">
-        <v>199.3242543587107</v>
+        <v>199.1462918111721</v>
       </c>
       <c r="K39" t="n">
-        <v>0.1236912055260483</v>
-      </c>
-      <c r="L39" t="inlineStr"/>
+        <v>0.1211556611899457</v>
+      </c>
+      <c r="L39" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M39" t="n">
         <v>182.2222222222222</v>
       </c>
@@ -3463,12 +3539,14 @@
         <v>165.7522199768573</v>
       </c>
       <c r="J40" t="n">
-        <v>199.6624849301809</v>
+        <v>199.5885882473661</v>
       </c>
       <c r="K40" t="n">
-        <v>0.1145922745262008</v>
-      </c>
-      <c r="L40" t="inlineStr"/>
+        <v>0.1159126568736139</v>
+      </c>
+      <c r="L40" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M40" t="n">
         <v>186.3157894736842</v>
       </c>
@@ -3539,12 +3617,14 @@
         <v>127.4617865350128</v>
       </c>
       <c r="J41" t="n">
-        <v>91.89362526827718</v>
+        <v>91.67853884817875</v>
       </c>
       <c r="K41" t="n">
-        <v>1.511609206255772</v>
-      </c>
-      <c r="L41" t="inlineStr"/>
+        <v>1.501031372391154</v>
+      </c>
+      <c r="L41" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M41" t="n">
         <v>183.507499093661</v>
       </c>
@@ -3617,12 +3697,14 @@
         <v>139.5371944473096</v>
       </c>
       <c r="J42" t="n">
-        <v>155.8038714031126</v>
+        <v>154.5839114750662</v>
       </c>
       <c r="K42" t="n">
-        <v>1.261630135771666</v>
-      </c>
-      <c r="L42" t="inlineStr"/>
+        <v>1.253514010486913</v>
+      </c>
+      <c r="L42" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M42" t="n">
         <v>181.2887708376975</v>
       </c>
@@ -3695,12 +3777,14 @@
         <v>137.8269504556986</v>
       </c>
       <c r="J43" t="n">
-        <v>129.0846217162649</v>
+        <v>129.2210590644231</v>
       </c>
       <c r="K43" t="n">
-        <v>0.8697344172166692</v>
-      </c>
-      <c r="L43" t="inlineStr"/>
+        <v>0.8683344472736246</v>
+      </c>
+      <c r="L43" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M43" t="n">
         <v>186.9457477180321</v>
       </c>
@@ -3773,12 +3857,14 @@
         <v>101.902133963665</v>
       </c>
       <c r="J44" t="n">
-        <v>113.9440981841071</v>
+        <v>113.6529259973059</v>
       </c>
       <c r="K44" t="n">
-        <v>1.94968755914931</v>
-      </c>
-      <c r="L44" t="inlineStr"/>
+        <v>1.94118931811028</v>
+      </c>
+      <c r="L44" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M44" t="n">
         <v>185.0623623920618</v>
       </c>
@@ -3851,12 +3937,14 @@
         <v>133.2410714461222</v>
       </c>
       <c r="J45" t="n">
-        <v>138.7678816808106</v>
+        <v>138.8865780666307</v>
       </c>
       <c r="K45" t="n">
-        <v>1.468288778039868</v>
-      </c>
-      <c r="L45" t="inlineStr"/>
+        <v>1.465205468677794</v>
+      </c>
+      <c r="L45" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M45" t="n">
         <v>181.9877754532652</v>
       </c>
@@ -3929,12 +4017,14 @@
         <v>129.1401202444324</v>
       </c>
       <c r="J46" t="n">
-        <v>154.2493653257513</v>
+        <v>155.5388593759895</v>
       </c>
       <c r="K46" t="n">
-        <v>1.085230101094652</v>
-      </c>
-      <c r="L46" t="inlineStr"/>
+        <v>1.100678491829755</v>
+      </c>
+      <c r="L46" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M46" t="n">
         <v>187.2242110784918</v>
       </c>
@@ -4007,12 +4097,14 @@
         <v>52.02932925897922</v>
       </c>
       <c r="J47" t="n">
-        <v>195.6050915352664</v>
+        <v>195.5685574757462</v>
       </c>
       <c r="K47" t="n">
-        <v>0.6016355901040529</v>
-      </c>
-      <c r="L47" t="inlineStr"/>
+        <v>0.5965869982198665</v>
+      </c>
+      <c r="L47" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M47" t="n">
         <v>198.4000634090768</v>
       </c>
@@ -4083,12 +4175,14 @@
         <v>75.82494372432545</v>
       </c>
       <c r="J48" t="n">
-        <v>198.5785629334108</v>
+        <v>198.5330491254405</v>
       </c>
       <c r="K48" t="n">
-        <v>0.208424441549574</v>
-      </c>
-      <c r="L48" t="inlineStr"/>
+        <v>0.2077539489681783</v>
+      </c>
+      <c r="L48" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M48" t="n">
         <v>197.2179224008849</v>
       </c>
@@ -4162,9 +4256,11 @@
         <v>200</v>
       </c>
       <c r="K49" t="n">
-        <v>0.3455497331267909</v>
-      </c>
-      <c r="L49" t="inlineStr"/>
+        <v>0.3437848424462895</v>
+      </c>
+      <c r="L49" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M49" t="n">
         <v>200</v>
       </c>
@@ -4235,12 +4331,14 @@
         <v>162.6912701840232</v>
       </c>
       <c r="J50" t="n">
-        <v>199.5122170374651</v>
+        <v>199.5486379903699</v>
       </c>
       <c r="K50" t="n">
-        <v>0.1641351663989946</v>
-      </c>
-      <c r="L50" t="inlineStr"/>
+        <v>0.1629152076573967</v>
+      </c>
+      <c r="L50" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M50" t="n">
         <v>200</v>
       </c>
@@ -4311,12 +4409,14 @@
         <v>169.9274838481079</v>
       </c>
       <c r="J51" t="n">
-        <v>199.569745356571</v>
+        <v>199.4865823478398</v>
       </c>
       <c r="K51" t="n">
-        <v>0.1221110404092794</v>
-      </c>
-      <c r="L51" t="inlineStr"/>
+        <v>0.1279910504674757</v>
+      </c>
+      <c r="L51" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M51" t="n">
         <v>195.959595959596</v>
       </c>
@@ -4387,12 +4487,14 @@
         <v>174.432365021141</v>
       </c>
       <c r="J52" t="n">
-        <v>199.8419507455721</v>
+        <v>199.8575276644268</v>
       </c>
       <c r="K52" t="n">
-        <v>0.06365527772305327</v>
-      </c>
-      <c r="L52" t="inlineStr"/>
+        <v>0.06289546852160235</v>
+      </c>
+      <c r="L52" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M52" t="n">
         <v>196.6386554621849</v>
       </c>
@@ -4463,12 +4565,14 @@
         <v>35.23746831954708</v>
       </c>
       <c r="J53" t="n">
-        <v>20.3485721220649</v>
+        <v>20.44901503425639</v>
       </c>
       <c r="K53" t="n">
-        <v>22.35766299143393</v>
-      </c>
-      <c r="L53" t="inlineStr"/>
+        <v>22.53472728636974</v>
+      </c>
+      <c r="L53" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M53" t="n">
         <v>162.1656348846054</v>
       </c>
@@ -4541,12 +4645,14 @@
         <v>38.4591918317379</v>
       </c>
       <c r="J54" t="n">
-        <v>21.4311848091815</v>
+        <v>21.5307402945977</v>
       </c>
       <c r="K54" t="n">
-        <v>11.31461757696774</v>
-      </c>
-      <c r="L54" t="inlineStr"/>
+        <v>11.37805163170186</v>
+      </c>
+      <c r="L54" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M54" t="n">
         <v>162.6260942449485</v>
       </c>
@@ -4576,11 +4682,11 @@
         </is>
       </c>
       <c r="U54" t="n">
-        <v>21.4311848091815</v>
+        <v>21.5307402945977</v>
       </c>
       <c r="V54" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=21.43% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=21.53% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4619,12 +4725,14 @@
         <v>38.25160771522186</v>
       </c>
       <c r="J55" t="n">
-        <v>23.44652230037202</v>
+        <v>23.26637498008379</v>
       </c>
       <c r="K55" t="n">
-        <v>13.31096246619567</v>
-      </c>
-      <c r="L55" t="inlineStr"/>
+        <v>13.17654509709004</v>
+      </c>
+      <c r="L55" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M55" t="n">
         <v>161.9773827308954</v>
       </c>
@@ -4654,11 +4762,11 @@
         </is>
       </c>
       <c r="U55" t="n">
-        <v>23.44652230037202</v>
+        <v>23.26637498008379</v>
       </c>
       <c r="V55" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=23.45% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=23.27% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4697,12 +4805,14 @@
         <v>154.1439500713238</v>
       </c>
       <c r="J56" t="n">
-        <v>60.29125449784342</v>
+        <v>60.38041763078138</v>
       </c>
       <c r="K56" t="n">
-        <v>2.058542600183989</v>
-      </c>
-      <c r="L56" t="inlineStr"/>
+        <v>2.065272317818089</v>
+      </c>
+      <c r="L56" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M56" t="n">
         <v>165.3708526408925</v>
       </c>
@@ -4732,11 +4842,11 @@
         </is>
       </c>
       <c r="U56" t="n">
-        <v>60.29125449784342</v>
+        <v>60.38041763078138</v>
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=60.29% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=60.38% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4775,12 +4885,14 @@
         <v>164.0555422208552</v>
       </c>
       <c r="J57" t="n">
-        <v>116.297575094597</v>
+        <v>114.7616231997743</v>
       </c>
       <c r="K57" t="n">
-        <v>1.527704620497148</v>
-      </c>
-      <c r="L57" t="inlineStr"/>
+        <v>1.488718622791548</v>
+      </c>
+      <c r="L57" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M57" t="n">
         <v>163.4899500853628</v>
       </c>
@@ -4853,12 +4965,14 @@
         <v>158.4722608607674</v>
       </c>
       <c r="J58" t="n">
-        <v>108.3078562554235</v>
+        <v>105.6303668976963</v>
       </c>
       <c r="K58" t="n">
-        <v>1.695960225704595</v>
-      </c>
-      <c r="L58" t="inlineStr"/>
+        <v>1.579491473670759</v>
+      </c>
+      <c r="L58" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M58" t="n">
         <v>167.6753221837887</v>
       </c>
@@ -4931,12 +5045,14 @@
         <v>163.442478475025</v>
       </c>
       <c r="J59" t="n">
-        <v>192.0282448335926</v>
+        <v>192.5368174319365</v>
       </c>
       <c r="K59" t="n">
-        <v>0.2176559100684902</v>
-      </c>
-      <c r="L59" t="inlineStr"/>
+        <v>0.2214133618233808</v>
+      </c>
+      <c r="L59" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M59" t="n">
         <v>171.7647058823529</v>
       </c>
@@ -5007,12 +5123,14 @@
         <v>179.6544870721095</v>
       </c>
       <c r="J60" t="n">
-        <v>198.0983117983889</v>
+        <v>198.6597355840884</v>
       </c>
       <c r="K60" t="n">
-        <v>0.1643773387814032</v>
-      </c>
-      <c r="L60" t="inlineStr"/>
+        <v>0.1659645822432419</v>
+      </c>
+      <c r="L60" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M60" t="n">
         <v>163.0769230769231</v>
       </c>
@@ -5083,12 +5201,14 @@
         <v>178.3754768379913</v>
       </c>
       <c r="J61" t="n">
-        <v>198.6805210475813</v>
+        <v>198.3975506268872</v>
       </c>
       <c r="K61" t="n">
-        <v>0.1343820781330749</v>
-      </c>
-      <c r="L61" t="inlineStr"/>
+        <v>0.137526459316728</v>
+      </c>
+      <c r="L61" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M61" t="n">
         <v>185.4545454545454</v>
       </c>
@@ -5159,12 +5279,14 @@
         <v>51.86246745886869</v>
       </c>
       <c r="J62" t="n">
-        <v>130.9571266908071</v>
+        <v>131.2644356700371</v>
       </c>
       <c r="K62" t="n">
-        <v>1.758318531644439</v>
-      </c>
-      <c r="L62" t="inlineStr"/>
+        <v>1.792143665152412</v>
+      </c>
+      <c r="L62" t="n">
+        <v>109.609711216533</v>
+      </c>
       <c r="M62" t="n">
         <v>175.5235927343014</v>
       </c>
@@ -5237,12 +5359,14 @@
         <v>69.84803023883232</v>
       </c>
       <c r="J63" t="n">
-        <v>160.7230440211508</v>
+        <v>160.5762472922584</v>
       </c>
       <c r="K63" t="n">
-        <v>0.4234746267679511</v>
-      </c>
-      <c r="L63" t="inlineStr"/>
+        <v>0.4223166429292686</v>
+      </c>
+      <c r="L63" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M63" t="n">
         <v>176.4842587752804</v>
       </c>
@@ -5313,12 +5437,14 @@
         <v>72.92360982323459</v>
       </c>
       <c r="J64" t="n">
-        <v>166.1274744316233</v>
+        <v>165.4971729021378</v>
       </c>
       <c r="K64" t="n">
-        <v>0.5598670879556945</v>
-      </c>
-      <c r="L64" t="inlineStr"/>
+        <v>0.5568628189725624</v>
+      </c>
+      <c r="L64" t="n">
+        <v>109.7635513825217</v>
+      </c>
       <c r="M64" t="n">
         <v>176.5775401069519</v>
       </c>
@@ -5389,10 +5515,10 @@
         <v>124.1398173354868</v>
       </c>
       <c r="J65" t="n">
-        <v>189.1042820076799</v>
+        <v>188.6285607672464</v>
       </c>
       <c r="K65" t="n">
-        <v>0.3797058234358746</v>
+        <v>0.3784678200407356</v>
       </c>
       <c r="L65" t="n">
         <v>137.6406301580537</v>
@@ -5467,12 +5593,14 @@
         <v>146.9871894171194</v>
       </c>
       <c r="J66" t="n">
-        <v>193.2101731341945</v>
+        <v>193.2466259789231</v>
       </c>
       <c r="K66" t="n">
-        <v>0.2751233810656595</v>
-      </c>
-      <c r="L66" t="inlineStr"/>
+        <v>0.2704853797460072</v>
+      </c>
+      <c r="L66" t="n">
+        <v>79.54507935933471</v>
+      </c>
       <c r="M66" t="n">
         <v>193.7098844672657</v>
       </c>
@@ -5543,10 +5671,10 @@
         <v>137.6516466078508</v>
       </c>
       <c r="J67" t="n">
-        <v>199.4595197986712</v>
+        <v>199.3097191502</v>
       </c>
       <c r="K67" t="n">
-        <v>0.2938794965819146</v>
+        <v>0.2915347690590922</v>
       </c>
       <c r="L67" t="n">
         <v>151.2037021887013</v>
@@ -5621,10 +5749,10 @@
         <v>183.5383709430125</v>
       </c>
       <c r="J68" t="n">
-        <v>199.8261929576067</v>
+        <v>199.7828034264477</v>
       </c>
       <c r="K68" t="n">
-        <v>0.0661948246945351</v>
+        <v>0.06645011343186964</v>
       </c>
       <c r="L68" t="n">
         <v>198.3312090033645</v>
@@ -5699,10 +5827,10 @@
         <v>171.5447439761989</v>
       </c>
       <c r="J69" t="n">
-        <v>199.4593995691129</v>
+        <v>199.3873217860459</v>
       </c>
       <c r="K69" t="n">
-        <v>0.07715776683387024</v>
+        <v>0.07890491428071096</v>
       </c>
       <c r="L69" t="n">
         <v>194.4182830751776</v>
@@ -5780,7 +5908,7 @@
         <v>200</v>
       </c>
       <c r="K70" t="n">
-        <v>0.01701156060708355</v>
+        <v>0.01611044537267105</v>
       </c>
       <c r="L70" t="n">
         <v>198.9765474653765</v>
@@ -5855,10 +5983,10 @@
         <v>143.4057585362926</v>
       </c>
       <c r="J71" t="n">
-        <v>181.7289735216879</v>
+        <v>181.9880034485936</v>
       </c>
       <c r="K71" t="n">
-        <v>4.204953221303974</v>
+        <v>4.205103676707298</v>
       </c>
       <c r="L71" t="n">
         <v>171.2174826415851</v>
@@ -5935,10 +6063,10 @@
         <v>151.0433307550491</v>
       </c>
       <c r="J72" t="n">
-        <v>96.98750299847268</v>
+        <v>97.00281078314966</v>
       </c>
       <c r="K72" t="n">
-        <v>1.305697114865129</v>
+        <v>1.286265630916457</v>
       </c>
       <c r="L72" t="n">
         <v>171.9287045593839</v>
@@ -6015,10 +6143,10 @@
         <v>148.5993365374143</v>
       </c>
       <c r="J73" t="n">
-        <v>167.6095784999177</v>
+        <v>167.6451026349307</v>
       </c>
       <c r="K73" t="n">
-        <v>2.325709697108638</v>
+        <v>2.318164934182062</v>
       </c>
       <c r="L73" t="n">
         <v>191.7880460732582</v>
@@ -6095,10 +6223,10 @@
         <v>148.9425712788151</v>
       </c>
       <c r="J74" t="n">
-        <v>186.9126864191641</v>
+        <v>187.0298527328072</v>
       </c>
       <c r="K74" t="n">
-        <v>0.4401064702641599</v>
+        <v>0.4419976246736432</v>
       </c>
       <c r="L74" t="n">
         <v>144.0733541161664</v>
@@ -6173,10 +6301,10 @@
         <v>157.2380343536269</v>
       </c>
       <c r="J75" t="n">
-        <v>196.6279104486694</v>
+        <v>196.6160780833582</v>
       </c>
       <c r="K75" t="n">
-        <v>0.3034072430596306</v>
+        <v>0.3031989103336238</v>
       </c>
       <c r="L75" t="n">
         <v>158.6014909691414</v>
@@ -6251,10 +6379,10 @@
         <v>154.9841830576604</v>
       </c>
       <c r="J76" t="n">
-        <v>195.3413856273902</v>
+        <v>195.1948412340681</v>
       </c>
       <c r="K76" t="n">
-        <v>0.2057436508728052</v>
+        <v>0.2055997108742528</v>
       </c>
       <c r="L76" t="n">
         <v>166.7038660732646</v>
@@ -6329,10 +6457,10 @@
         <v>77.76772218573589</v>
       </c>
       <c r="J77" t="n">
-        <v>36.79734774047761</v>
+        <v>37.10004537508804</v>
       </c>
       <c r="K77" t="n">
-        <v>6.708211027185509</v>
+        <v>6.776254930868525</v>
       </c>
       <c r="L77" t="n">
         <v>110.3330967959057</v>
@@ -6366,11 +6494,11 @@
         </is>
       </c>
       <c r="U77" t="n">
-        <v>36.79734774047761</v>
+        <v>37.10004537508804</v>
       </c>
       <c r="V77" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=36.80% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=37.10% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6409,10 +6537,10 @@
         <v>103.5437500854655</v>
       </c>
       <c r="J78" t="n">
-        <v>51.10941098137504</v>
+        <v>49.13942155356582</v>
       </c>
       <c r="K78" t="n">
-        <v>4.074518054301315</v>
+        <v>3.932447908708014</v>
       </c>
       <c r="L78" t="n">
         <v>115.3631910942854</v>
@@ -6489,10 +6617,10 @@
         <v>102.5016657415887</v>
       </c>
       <c r="J79" t="n">
-        <v>36.92725458042533</v>
+        <v>36.89186308680129</v>
       </c>
       <c r="K79" t="n">
-        <v>3.302047854258936</v>
+        <v>3.304314077057211</v>
       </c>
       <c r="L79" t="n">
         <v>114.5134591086363</v>
@@ -6526,11 +6654,11 @@
         </is>
       </c>
       <c r="U79" t="n">
-        <v>36.92725458042533</v>
+        <v>36.89186308680129</v>
       </c>
       <c r="V79" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=36.93% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=36.89% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6569,10 +6697,10 @@
         <v>180.9937478063148</v>
       </c>
       <c r="J80" t="n">
-        <v>149.3522092224518</v>
+        <v>148.3561506538706</v>
       </c>
       <c r="K80" t="n">
-        <v>23.38961870508665</v>
+        <v>23.31756395053142</v>
       </c>
       <c r="L80" t="n">
         <v>195.3549053278383</v>
@@ -6649,10 +6777,10 @@
         <v>185.5191244575439</v>
       </c>
       <c r="J81" t="n">
-        <v>135.1025520610708</v>
+        <v>137.2064188235088</v>
       </c>
       <c r="K81" t="n">
-        <v>8.567143251050577</v>
+        <v>8.59187932191203</v>
       </c>
       <c r="L81" t="n">
         <v>199.4307199889832</v>
@@ -6729,10 +6857,10 @@
         <v>186.2973802760101</v>
       </c>
       <c r="J82" t="n">
-        <v>143.6520875442592</v>
+        <v>145.1472793964314</v>
       </c>
       <c r="K82" t="n">
-        <v>12.94659064734331</v>
+        <v>12.99796069573456</v>
       </c>
       <c r="L82" t="n">
         <v>183.0162368876618</v>
@@ -6809,10 +6937,10 @@
         <v>88.04980557911651</v>
       </c>
       <c r="J83" t="n">
-        <v>46.42585692650886</v>
+        <v>47.56092545874292</v>
       </c>
       <c r="K83" t="n">
-        <v>8.37710047108553</v>
+        <v>8.665217789405114</v>
       </c>
       <c r="L83" t="n">
         <v>194.0620340843763</v>
@@ -6889,10 +7017,10 @@
         <v>100.4914466151705</v>
       </c>
       <c r="J84" t="n">
-        <v>45.96231344597865</v>
+        <v>46.15812962490158</v>
       </c>
       <c r="K84" t="n">
-        <v>3.449044160724878</v>
+        <v>3.475128502119654</v>
       </c>
       <c r="L84" t="n">
         <v>161.0256208848398</v>
@@ -6969,10 +7097,10 @@
         <v>109.9471447641292</v>
       </c>
       <c r="J85" t="n">
-        <v>57.43339810358206</v>
+        <v>55.36256686407579</v>
       </c>
       <c r="K85" t="n">
-        <v>5.058339965311367</v>
+        <v>4.933087742300096</v>
       </c>
       <c r="L85" t="n">
         <v>191.126671844217</v>
@@ -7049,10 +7177,10 @@
         <v>160.3842205944857</v>
       </c>
       <c r="J86" t="n">
-        <v>118.5283012694314</v>
+        <v>119.2256744546712</v>
       </c>
       <c r="K86" t="n">
-        <v>1.511365094958628</v>
+        <v>1.526445464584329</v>
       </c>
       <c r="L86" t="n">
         <v>143.9950818237897</v>
@@ -7129,10 +7257,10 @@
         <v>171.410316416684</v>
       </c>
       <c r="J87" t="n">
-        <v>143.5835389914779</v>
+        <v>143.560216889931</v>
       </c>
       <c r="K87" t="n">
-        <v>0.9800779156337266</v>
+        <v>0.9883869165511783</v>
       </c>
       <c r="L87" t="n">
         <v>150.2517475184781</v>
@@ -7209,10 +7337,10 @@
         <v>169.0038464611843</v>
       </c>
       <c r="J88" t="n">
-        <v>173.8296114884862</v>
+        <v>173.3382025272879</v>
       </c>
       <c r="K88" t="n">
-        <v>1.003422029570916</v>
+        <v>1.000072263696867</v>
       </c>
       <c r="L88" t="n">
         <v>118.6804789630648</v>
@@ -7292,7 +7420,7 @@
         <v>200</v>
       </c>
       <c r="K89" t="n">
-        <v>0.007380532391221194</v>
+        <v>0.007270478566362362</v>
       </c>
       <c r="L89" t="n">
         <v>200</v>
@@ -7366,7 +7494,7 @@
         <v>200</v>
       </c>
       <c r="K90" t="n">
-        <v>0.003657128813195968</v>
+        <v>0.003415887464000547</v>
       </c>
       <c r="L90" t="n">
         <v>200</v>
@@ -7440,7 +7568,7 @@
         <v>200</v>
       </c>
       <c r="K91" t="n">
-        <v>0.01455603600441123</v>
+        <v>0.01376589551061007</v>
       </c>
       <c r="L91" t="n">
         <v>200</v>
@@ -7511,10 +7639,10 @@
         <v>49.15109590531281</v>
       </c>
       <c r="J92" t="n">
-        <v>53.35077005079972</v>
+        <v>53.86994196900773</v>
       </c>
       <c r="K92" t="n">
-        <v>7.637694966892938</v>
+        <v>7.694847947284689</v>
       </c>
       <c r="L92" t="n">
         <v>104.6459551741298</v>
@@ -7591,10 +7719,10 @@
         <v>60.93105560683724</v>
       </c>
       <c r="J93" t="n">
-        <v>60.1026346278737</v>
+        <v>59.78155232420327</v>
       </c>
       <c r="K93" t="n">
-        <v>4.939438714442002</v>
+        <v>4.925424425520819</v>
       </c>
       <c r="L93" t="n">
         <v>89.5280086489867</v>
@@ -7671,10 +7799,10 @@
         <v>64.07712599234655</v>
       </c>
       <c r="J94" t="n">
-        <v>52.98096764410323</v>
+        <v>52.69581648158714</v>
       </c>
       <c r="K94" t="n">
-        <v>3.790476368256205</v>
+        <v>3.740125253417435</v>
       </c>
       <c r="L94" t="n">
         <v>91.94886769427217</v>
@@ -7708,11 +7836,11 @@
         </is>
       </c>
       <c r="U94" t="n">
-        <v>52.98096764410323</v>
+        <v>52.69581648158714</v>
       </c>
       <c r="V94" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=52.98% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=52.70% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7751,10 +7879,10 @@
         <v>152.3875262412586</v>
       </c>
       <c r="J95" t="n">
-        <v>198.9660683083715</v>
+        <v>199.1922050178509</v>
       </c>
       <c r="K95" t="n">
-        <v>0.5239013555859853</v>
+        <v>0.5243681068222776</v>
       </c>
       <c r="L95" t="n">
         <v>128.1095321097334</v>
@@ -7831,10 +7959,10 @@
         <v>158.9896824444987</v>
       </c>
       <c r="J96" t="n">
-        <v>199.2150951603351</v>
+        <v>199.2513153043118</v>
       </c>
       <c r="K96" t="n">
-        <v>0.1584986195278356</v>
+        <v>0.158291047634362</v>
       </c>
       <c r="L96" t="n">
         <v>189.1617640516506</v>
@@ -7909,10 +8037,10 @@
         <v>157.2976315063829</v>
       </c>
       <c r="J97" t="n">
-        <v>199.3927310976356</v>
+        <v>199.3614643125625</v>
       </c>
       <c r="K97" t="n">
-        <v>0.3716897725749284</v>
+        <v>0.3712739720909262</v>
       </c>
       <c r="L97" t="n">
         <v>187.1093440450062</v>
@@ -7990,7 +8118,7 @@
         <v>200</v>
       </c>
       <c r="K98" t="n">
-        <v>0.0005744433579079894</v>
+        <v>0.000548695229506579</v>
       </c>
       <c r="L98" t="n">
         <v>199.9898962083731</v>
@@ -8064,7 +8192,7 @@
         <v>200</v>
       </c>
       <c r="K99" t="n">
-        <v>0.001595394861881958</v>
+        <v>0.001607453320843158</v>
       </c>
       <c r="L99" t="n">
         <v>199.9983019911245</v>
@@ -8138,7 +8266,7 @@
         <v>200</v>
       </c>
       <c r="K100" t="n">
-        <v>0.00240448959164621</v>
+        <v>0.002433839398527311</v>
       </c>
       <c r="L100" t="n">
         <v>200</v>

</xml_diff>

<commit_message>
feat(dengue): ENSO Prophet en producción + reselect (nacional->DeepAR, dist 56/43)
- Re-entrenadas las 99 series Prophet Dengue con el regresor El Niño/ONI; reselect
  produccion_dengue: distribución DeepAR 56 / Prophet 43, Nacional=DeepAR.
- El ENSO Prophet anticipa más magnitud (validado en años epidémicos: SMAPE 2024
  62->31); en 2026 (año bajo) eso sube su SMAPE-real nacional 20.3->23.2 y cede el
  nacional a DeepAR (SMAPE 20.4, forecast 52sem 23,832 vs el viejo Prophet sub-predecía 13k).
- model.py: _attach_enso usa copias (evita SettingWithCopyWarning). 73 tests OK.
- NEURO INTACTO: forecasts neuro byte-idénticos (yhat sum verificado), reselect solo Dengue.
</commit_message>
<xml_diff>
--- a/reports/ProdDetails/produccion_dengue.xlsx
+++ b/reports/ProdDetails/produccion_dengue.xlsx
@@ -569,10 +569,10 @@
         <v>200</v>
       </c>
       <c r="H2" t="n">
-        <v>0.01143971376208275</v>
+        <v>0.01909339069720435</v>
       </c>
       <c r="I2" t="n">
-        <v>185.8333489727328</v>
+        <v>181.8875746538405</v>
       </c>
       <c r="J2" t="n">
         <v>200</v>
@@ -647,10 +647,10 @@
         <v>200</v>
       </c>
       <c r="H3" t="n">
-        <v>0.009067953039092178</v>
+        <v>0.0120984434586246</v>
       </c>
       <c r="I3" t="n">
-        <v>157.2321783542833</v>
+        <v>157.3839857426704</v>
       </c>
       <c r="J3" t="n">
         <v>200</v>
@@ -725,10 +725,10 @@
         <v>200</v>
       </c>
       <c r="H4" t="n">
-        <v>0.01410237981501257</v>
+        <v>0.02123577474837053</v>
       </c>
       <c r="I4" t="n">
-        <v>158.5580779411727</v>
+        <v>158.8438418444702</v>
       </c>
       <c r="J4" t="n">
         <v>200</v>
@@ -800,13 +800,13 @@
         <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>199.0125831330724</v>
+        <v>199.863029343531</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1083988208702625</v>
+        <v>0.1060038941382352</v>
       </c>
       <c r="I5" t="n">
-        <v>175.1088701866436</v>
+        <v>175.5400786038201</v>
       </c>
       <c r="J5" t="n">
         <v>199.2843630995856</v>
@@ -878,13 +878,13 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>199.5227768499908</v>
+        <v>199.6986714004902</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06224017002961615</v>
+        <v>0.05880289809912526</v>
       </c>
       <c r="I6" t="n">
-        <v>191.646475967384</v>
+        <v>191.737797552366</v>
       </c>
       <c r="J6" t="n">
         <v>199.9861671147559</v>
@@ -956,13 +956,13 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>199.0827646374914</v>
+        <v>199.158331088558</v>
       </c>
       <c r="H7" t="n">
-        <v>0.07542585392837421</v>
+        <v>0.06346581821336009</v>
       </c>
       <c r="I7" t="n">
-        <v>186.9197740801393</v>
+        <v>187.2671055681853</v>
       </c>
       <c r="J7" t="n">
         <v>199.9884309380623</v>
@@ -1034,13 +1034,13 @@
         <v>142</v>
       </c>
       <c r="G8" t="n">
-        <v>101.1620929265983</v>
+        <v>124.2408629147414</v>
       </c>
       <c r="H8" t="n">
-        <v>5.212131266542356</v>
+        <v>5.858449498066894</v>
       </c>
       <c r="I8" t="n">
-        <v>154.5040916050135</v>
+        <v>146.1852288200182</v>
       </c>
       <c r="J8" t="n">
         <v>48.2035225269852</v>
@@ -1114,13 +1114,13 @@
         <v>62</v>
       </c>
       <c r="G9" t="n">
-        <v>96.50000967408079</v>
+        <v>133.862958905723</v>
       </c>
       <c r="H9" t="n">
-        <v>2.364058607609518</v>
+        <v>2.745953184050532</v>
       </c>
       <c r="I9" t="n">
-        <v>164.086229256472</v>
+        <v>155.2184985113495</v>
       </c>
       <c r="J9" t="n">
         <v>69.98966250353146</v>
@@ -1194,13 +1194,13 @@
         <v>75</v>
       </c>
       <c r="G10" t="n">
-        <v>94.84727283752737</v>
+        <v>124.9117102132738</v>
       </c>
       <c r="H10" t="n">
-        <v>2.632141656550983</v>
+        <v>3.060920355992553</v>
       </c>
       <c r="I10" t="n">
-        <v>164.4874496413386</v>
+        <v>152.9918981156764</v>
       </c>
       <c r="J10" t="n">
         <v>45.23277359273659</v>
@@ -1274,13 +1274,13 @@
         <v>11</v>
       </c>
       <c r="G11" t="n">
-        <v>177.1662152513658</v>
+        <v>169.256431894795</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5816049116984011</v>
+        <v>0.5989329700208699</v>
       </c>
       <c r="I11" t="n">
-        <v>123.2554563734294</v>
+        <v>129.9250091591691</v>
       </c>
       <c r="J11" t="n">
         <v>198.0164154965292</v>
@@ -1320,11 +1320,11 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>177.1662152513658</v>
+        <v>169.256431894795</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=177.17% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=169.26% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1354,13 +1354,13 @@
         <v>7</v>
       </c>
       <c r="G12" t="n">
-        <v>191.8552562166053</v>
+        <v>194.4159379304537</v>
       </c>
       <c r="H12" t="n">
-        <v>0.3754643963600293</v>
+        <v>0.3858136158142387</v>
       </c>
       <c r="I12" t="n">
-        <v>147.3485671696691</v>
+        <v>140.9543563511172</v>
       </c>
       <c r="J12" t="n">
         <v>199.523179310629</v>
@@ -1432,13 +1432,13 @@
         <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>195.3735385790647</v>
+        <v>194.7808770000501</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2165418703011477</v>
+        <v>0.2470576173028503</v>
       </c>
       <c r="I13" t="n">
-        <v>157.1522264328246</v>
+        <v>143.0465384202982</v>
       </c>
       <c r="J13" t="n">
         <v>199.8262982460481</v>
@@ -1510,13 +1510,13 @@
         <v>62</v>
       </c>
       <c r="G14" t="n">
-        <v>70.98011798172448</v>
+        <v>68.18440924623016</v>
       </c>
       <c r="H14" t="n">
-        <v>2.050209983850287</v>
+        <v>1.965115005649187</v>
       </c>
       <c r="I14" t="n">
-        <v>66.61025297793201</v>
+        <v>74.93132855047638</v>
       </c>
       <c r="J14" t="n">
         <v>85.47396170872173</v>
@@ -1556,11 +1556,11 @@
         </is>
       </c>
       <c r="U14" t="n">
-        <v>70.98011798172448</v>
+        <v>68.18440924623016</v>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=70.98% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=68.18% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1590,13 +1590,13 @@
         <v>32</v>
       </c>
       <c r="G15" t="n">
-        <v>65.87044566451193</v>
+        <v>68.63649638136945</v>
       </c>
       <c r="H15" t="n">
-        <v>0.897248034177942</v>
+        <v>0.9654501657857059</v>
       </c>
       <c r="I15" t="n">
-        <v>82.6747998505866</v>
+        <v>83.26703869122109</v>
       </c>
       <c r="J15" t="n">
         <v>89.8785759618037</v>
@@ -1636,11 +1636,11 @@
         </is>
       </c>
       <c r="U15" t="n">
-        <v>65.87044566451193</v>
+        <v>68.63649638136945</v>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=65.87% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=68.64% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1670,13 +1670,13 @@
         <v>30</v>
       </c>
       <c r="G16" t="n">
-        <v>122.3179070028762</v>
+        <v>121.4424954946124</v>
       </c>
       <c r="H16" t="n">
-        <v>1.567952396243824</v>
+        <v>1.534736430505168</v>
       </c>
       <c r="I16" t="n">
-        <v>90.20708978859948</v>
+        <v>88.28301425252694</v>
       </c>
       <c r="J16" t="n">
         <v>142.02923967689</v>
@@ -1716,11 +1716,11 @@
         </is>
       </c>
       <c r="U16" t="n">
-        <v>122.3179070028762</v>
+        <v>121.4424954946124</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=122.32% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=121.44% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1750,13 +1750,13 @@
         <v>1</v>
       </c>
       <c r="G17" t="n">
-        <v>198.7352626872857</v>
+        <v>199.1102341795934</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1117349335808297</v>
+        <v>0.09613834946315496</v>
       </c>
       <c r="I17" t="n">
-        <v>194.5446671655584</v>
+        <v>194.6710344353644</v>
       </c>
       <c r="J17" t="n">
         <v>199.943152462609</v>
@@ -1831,10 +1831,10 @@
         <v>200</v>
       </c>
       <c r="H18" t="n">
-        <v>0.02565291991697691</v>
+        <v>0.03136352411444188</v>
       </c>
       <c r="I18" t="n">
-        <v>199.6410247115898</v>
+        <v>199.5917940260522</v>
       </c>
       <c r="J18" t="n">
         <v>200</v>
@@ -1902,13 +1902,13 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>199.0372771487083</v>
+        <v>199.4476600573335</v>
       </c>
       <c r="H19" t="n">
-        <v>0.09944267109328039</v>
+        <v>0.08682774457069804</v>
       </c>
       <c r="I19" t="n">
-        <v>196.278530387405</v>
+        <v>196.3668815794815</v>
       </c>
       <c r="J19" t="n">
         <v>199.8695191024682</v>
@@ -1983,7 +1983,7 @@
         <v>200</v>
       </c>
       <c r="H20" t="n">
-        <v>0.07047412404518942</v>
+        <v>0.01308918116114505</v>
       </c>
       <c r="I20" t="n">
         <v>200</v>
@@ -2057,7 +2057,7 @@
         <v>200</v>
       </c>
       <c r="H21" t="n">
-        <v>0.05672395709071366</v>
+        <v>0.05679447572271468</v>
       </c>
       <c r="I21" t="n">
         <v>200</v>
@@ -2131,7 +2131,7 @@
         <v>200</v>
       </c>
       <c r="H22" t="n">
-        <v>0.06350447684539688</v>
+        <v>0.06271867433330723</v>
       </c>
       <c r="I22" t="n">
         <v>200</v>
@@ -2202,13 +2202,13 @@
         <v>2</v>
       </c>
       <c r="G23" t="n">
-        <v>179.1739130190571</v>
+        <v>179.9337722008812</v>
       </c>
       <c r="H23" t="n">
-        <v>0.1271859159213902</v>
+        <v>0.1264170913622294</v>
       </c>
       <c r="I23" t="n">
-        <v>149.2565324185079</v>
+        <v>148.7957871310144</v>
       </c>
       <c r="J23" t="n">
         <v>199.2619412956352</v>
@@ -2280,13 +2280,13 @@
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>182.221104530061</v>
+        <v>182.6845580141106</v>
       </c>
       <c r="H24" t="n">
-        <v>0.06574743966708289</v>
+        <v>0.06542854972043259</v>
       </c>
       <c r="I24" t="n">
-        <v>156.2502876793226</v>
+        <v>155.1760639717555</v>
       </c>
       <c r="J24" t="n">
         <v>198.5231057940479</v>
@@ -2361,10 +2361,10 @@
         <v>200</v>
       </c>
       <c r="H25" t="n">
-        <v>0.0735937728171784</v>
+        <v>0.07054487750177577</v>
       </c>
       <c r="I25" t="n">
-        <v>155.3955473497874</v>
+        <v>155.0685899856278</v>
       </c>
       <c r="J25" t="n">
         <v>199.9139299449369</v>
@@ -2439,10 +2439,10 @@
         <v>200</v>
       </c>
       <c r="H26" t="n">
-        <v>0.02780046601968817</v>
+        <v>0.0832718885486983</v>
       </c>
       <c r="I26" t="n">
-        <v>97.19414576199205</v>
+        <v>109.9617469881321</v>
       </c>
       <c r="J26" t="n">
         <v>200</v>
@@ -2517,10 +2517,10 @@
         <v>200</v>
       </c>
       <c r="H27" t="n">
-        <v>0.01946588280507898</v>
+        <v>0.004602625390390047</v>
       </c>
       <c r="I27" t="n">
-        <v>129.0985231723771</v>
+        <v>128.3332125535668</v>
       </c>
       <c r="J27" t="n">
         <v>200</v>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>DeepAR</t>
+          <t>Prophet</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
@@ -2562,7 +2562,7 @@
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr">
         <is>
-          <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
+          <t>Prophet: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -2595,10 +2595,10 @@
         <v>200</v>
       </c>
       <c r="H28" t="n">
-        <v>0.01964014595132009</v>
+        <v>0.02779200000818176</v>
       </c>
       <c r="I28" t="n">
-        <v>127.1718885128103</v>
+        <v>134.8536674445885</v>
       </c>
       <c r="J28" t="n">
         <v>200</v>
@@ -2673,10 +2673,10 @@
         <v>200</v>
       </c>
       <c r="H29" t="n">
-        <v>0.09615446603845537</v>
+        <v>0.1866389784049496</v>
       </c>
       <c r="I29" t="n">
-        <v>191.5075017030775</v>
+        <v>192.4134519048118</v>
       </c>
       <c r="J29" t="n">
         <v>200</v>
@@ -2751,10 +2751,10 @@
         <v>200</v>
       </c>
       <c r="H30" t="n">
-        <v>0.08151387564442503</v>
+        <v>0.1380433323432018</v>
       </c>
       <c r="I30" t="n">
-        <v>196.0386411854094</v>
+        <v>196.3947851007668</v>
       </c>
       <c r="J30" t="n">
         <v>200</v>
@@ -2829,10 +2829,10 @@
         <v>200</v>
       </c>
       <c r="H31" t="n">
-        <v>0.09432961679395827</v>
+        <v>0.1477795792688235</v>
       </c>
       <c r="I31" t="n">
-        <v>194.2466814459454</v>
+        <v>194.2709642910985</v>
       </c>
       <c r="J31" t="n">
         <v>200</v>
@@ -2904,13 +2904,13 @@
         <v>7</v>
       </c>
       <c r="G32" t="n">
-        <v>167.192582466706</v>
+        <v>165.7546148305496</v>
       </c>
       <c r="H32" t="n">
-        <v>0.3731776944879054</v>
+        <v>0.38785922921792</v>
       </c>
       <c r="I32" t="n">
-        <v>164.6748490827784</v>
+        <v>164.8758692530674</v>
       </c>
       <c r="J32" t="n">
         <v>188.3994774916149</v>
@@ -2985,10 +2985,10 @@
         <v>200</v>
       </c>
       <c r="H33" t="n">
-        <v>0.156967795367359</v>
+        <v>0.1535755243341698</v>
       </c>
       <c r="I33" t="n">
-        <v>170.4028696730483</v>
+        <v>170.1482256075269</v>
       </c>
       <c r="J33" t="n">
         <v>197.5602748361831</v>
@@ -3060,13 +3060,13 @@
         <v>6</v>
       </c>
       <c r="G34" t="n">
-        <v>175.6265418068303</v>
+        <v>174.6879222141001</v>
       </c>
       <c r="H34" t="n">
-        <v>0.3116447449667569</v>
+        <v>0.3296184931025303</v>
       </c>
       <c r="I34" t="n">
-        <v>169.6571057340244</v>
+        <v>171.4397998821392</v>
       </c>
       <c r="J34" t="n">
         <v>171.6084043022315</v>
@@ -3138,13 +3138,13 @@
         <v>15</v>
       </c>
       <c r="G35" t="n">
-        <v>105.0282170767762</v>
+        <v>108.3601558982242</v>
       </c>
       <c r="H35" t="n">
-        <v>0.6403055072847207</v>
+        <v>0.9926778426100719</v>
       </c>
       <c r="I35" t="n">
-        <v>48.55849570822402</v>
+        <v>62.42552765573187</v>
       </c>
       <c r="J35" t="n">
         <v>128.6246318422078</v>
@@ -3184,11 +3184,11 @@
         </is>
       </c>
       <c r="U35" t="n">
-        <v>105.0282170767762</v>
+        <v>108.3601558982242</v>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=105.03% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=108.36% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3218,13 +3218,13 @@
         <v>6</v>
       </c>
       <c r="G36" t="n">
-        <v>161.9953762443956</v>
+        <v>156.7844328162785</v>
       </c>
       <c r="H36" t="n">
-        <v>0.4122286060260453</v>
+        <v>0.6980743927875586</v>
       </c>
       <c r="I36" t="n">
-        <v>58.86670393327421</v>
+        <v>70.10918162979605</v>
       </c>
       <c r="J36" t="n">
         <v>170.6440396621451</v>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>DeepAR</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
@@ -3266,7 +3266,7 @@
       <c r="U36" t="inlineStr"/>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Prophet: serie casi-cero (total 6 casos), menor MAE real</t>
+          <t>DeepAR: serie casi-cero (total 6 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -3296,13 +3296,13 @@
         <v>9</v>
       </c>
       <c r="G37" t="n">
-        <v>149.3030044507669</v>
+        <v>142.6549908394647</v>
       </c>
       <c r="H37" t="n">
-        <v>0.6340439810854436</v>
+        <v>0.7294146855502518</v>
       </c>
       <c r="I37" t="n">
-        <v>60.32903496111531</v>
+        <v>69.25953978081323</v>
       </c>
       <c r="J37" t="n">
         <v>162.0004203901676</v>
@@ -3374,13 +3374,13 @@
         <v>4</v>
       </c>
       <c r="G38" t="n">
-        <v>191.9919619009012</v>
+        <v>199.6217616830302</v>
       </c>
       <c r="H38" t="n">
-        <v>0.4533242349898883</v>
+        <v>0.3370447620534833</v>
       </c>
       <c r="I38" t="n">
-        <v>164.4263244057969</v>
+        <v>162.149087371204</v>
       </c>
       <c r="J38" t="n">
         <v>193.5392151146532</v>
@@ -3452,13 +3452,13 @@
         <v>2</v>
       </c>
       <c r="G39" t="n">
-        <v>198.5118901369247</v>
+        <v>200</v>
       </c>
       <c r="H39" t="n">
-        <v>0.1737669757217708</v>
+        <v>0.1285627026425347</v>
       </c>
       <c r="I39" t="n">
-        <v>170.2041702191862</v>
+        <v>165.7621571068165</v>
       </c>
       <c r="J39" t="n">
         <v>199.1462918111721</v>
@@ -3530,13 +3530,13 @@
         <v>2</v>
       </c>
       <c r="G40" t="n">
-        <v>197.8503046852848</v>
+        <v>200</v>
       </c>
       <c r="H40" t="n">
-        <v>0.2175630299201529</v>
+        <v>0.1607786834568675</v>
       </c>
       <c r="I40" t="n">
-        <v>165.7522199768573</v>
+        <v>163.618905219222</v>
       </c>
       <c r="J40" t="n">
         <v>199.5885882473661</v>
@@ -3608,13 +3608,13 @@
         <v>47</v>
       </c>
       <c r="G41" t="n">
-        <v>87.77044360060759</v>
+        <v>82.11866101265029</v>
       </c>
       <c r="H41" t="n">
-        <v>1.856873350730323</v>
+        <v>1.598833157227979</v>
       </c>
       <c r="I41" t="n">
-        <v>127.4617865350128</v>
+        <v>132.9108801179189</v>
       </c>
       <c r="J41" t="n">
         <v>91.67853884817875</v>
@@ -3654,11 +3654,11 @@
         </is>
       </c>
       <c r="U41" t="n">
-        <v>87.77044360060759</v>
+        <v>82.11866101265029</v>
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=87.77% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=82.12% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3688,13 +3688,13 @@
         <v>25</v>
       </c>
       <c r="G42" t="n">
-        <v>113.7548643964564</v>
+        <v>109.6033369316858</v>
       </c>
       <c r="H42" t="n">
-        <v>1.223731755047448</v>
+        <v>1.06863407789476</v>
       </c>
       <c r="I42" t="n">
-        <v>139.5371944473096</v>
+        <v>144.2379256407503</v>
       </c>
       <c r="J42" t="n">
         <v>154.5839114750662</v>
@@ -3734,11 +3734,11 @@
         </is>
       </c>
       <c r="U42" t="n">
-        <v>113.7548643964564</v>
+        <v>109.6033369316858</v>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=113.75% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=109.60% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3768,13 +3768,13 @@
         <v>22</v>
       </c>
       <c r="G43" t="n">
-        <v>91.31975786598234</v>
+        <v>87.61246286752178</v>
       </c>
       <c r="H43" t="n">
-        <v>0.9782084518115962</v>
+        <v>0.8606773829398876</v>
       </c>
       <c r="I43" t="n">
-        <v>137.8269504556986</v>
+        <v>143.2356557138082</v>
       </c>
       <c r="J43" t="n">
         <v>129.2210590644231</v>
@@ -3814,11 +3814,11 @@
         </is>
       </c>
       <c r="U43" t="n">
-        <v>91.31975786598234</v>
+        <v>87.61246286752178</v>
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=91.32% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=87.61% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3848,13 +3848,13 @@
         <v>44</v>
       </c>
       <c r="G44" t="n">
-        <v>101.541216978027</v>
+        <v>96.02426038457011</v>
       </c>
       <c r="H44" t="n">
-        <v>3.270011438578409</v>
+        <v>2.811469877005802</v>
       </c>
       <c r="I44" t="n">
-        <v>101.902133963665</v>
+        <v>90.69108260489389</v>
       </c>
       <c r="J44" t="n">
         <v>113.6529259973059</v>
@@ -3894,11 +3894,11 @@
         </is>
       </c>
       <c r="U44" t="n">
-        <v>101.541216978027</v>
+        <v>96.02426038457011</v>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=101.54% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=96.02% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3928,13 +3928,13 @@
         <v>27</v>
       </c>
       <c r="G45" t="n">
-        <v>116.1460451702141</v>
+        <v>102.4367406023931</v>
       </c>
       <c r="H45" t="n">
-        <v>2.564017877299051</v>
+        <v>1.47241398353088</v>
       </c>
       <c r="I45" t="n">
-        <v>133.2410714461222</v>
+        <v>133.3421874706413</v>
       </c>
       <c r="J45" t="n">
         <v>138.8865780666307</v>
@@ -3974,11 +3974,11 @@
         </is>
       </c>
       <c r="U45" t="n">
-        <v>116.1460451702141</v>
+        <v>102.4367406023931</v>
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=116.15% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=102.44% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4008,13 +4008,13 @@
         <v>17</v>
       </c>
       <c r="G46" t="n">
-        <v>140.3897249540533</v>
+        <v>134.8495847933821</v>
       </c>
       <c r="H46" t="n">
-        <v>2.53501087439491</v>
+        <v>1.94188163307336</v>
       </c>
       <c r="I46" t="n">
-        <v>129.1401202444324</v>
+        <v>124.5635906347636</v>
       </c>
       <c r="J46" t="n">
         <v>155.5388593759895</v>
@@ -4054,11 +4054,11 @@
         </is>
       </c>
       <c r="U46" t="n">
-        <v>140.3897249540533</v>
+        <v>134.8495847933821</v>
       </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=140.39% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=134.85% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4088,13 +4088,13 @@
         <v>2</v>
       </c>
       <c r="G47" t="n">
-        <v>195.9411133670229</v>
+        <v>197.1734011497229</v>
       </c>
       <c r="H47" t="n">
-        <v>0.1636167997295013</v>
+        <v>0.1529803815317455</v>
       </c>
       <c r="I47" t="n">
-        <v>52.02932925897922</v>
+        <v>68.7708518238762</v>
       </c>
       <c r="J47" t="n">
         <v>195.5685574757462</v>
@@ -4166,13 +4166,13 @@
         <v>2</v>
       </c>
       <c r="G48" t="n">
-        <v>197.4116289114259</v>
+        <v>198.4050298288979</v>
       </c>
       <c r="H48" t="n">
-        <v>0.1238703056407061</v>
+        <v>0.1142571312560468</v>
       </c>
       <c r="I48" t="n">
-        <v>75.82494372432545</v>
+        <v>86.09499988689549</v>
       </c>
       <c r="J48" t="n">
         <v>198.5330491254405</v>
@@ -4247,10 +4247,10 @@
         <v>200</v>
       </c>
       <c r="H49" t="n">
-        <v>0.02509264972644333</v>
+        <v>0.03928420848952716</v>
       </c>
       <c r="I49" t="n">
-        <v>67.54170898302603</v>
+        <v>78.24471458494588</v>
       </c>
       <c r="J49" t="n">
         <v>200</v>
@@ -4322,13 +4322,13 @@
         <v>2</v>
       </c>
       <c r="G50" t="n">
-        <v>194.3911602673957</v>
+        <v>195.8965903086375</v>
       </c>
       <c r="H50" t="n">
-        <v>1.518323311321763</v>
+        <v>1.219447449788111</v>
       </c>
       <c r="I50" t="n">
-        <v>162.6912701840232</v>
+        <v>165.7288014065556</v>
       </c>
       <c r="J50" t="n">
         <v>199.5486379903699</v>
@@ -4400,13 +4400,13 @@
         <v>1</v>
       </c>
       <c r="G51" t="n">
-        <v>194.7647831852421</v>
+        <v>197.4072044927651</v>
       </c>
       <c r="H51" t="n">
-        <v>0.7618632865622107</v>
+        <v>0.5937166551583655</v>
       </c>
       <c r="I51" t="n">
-        <v>169.9274838481079</v>
+        <v>167.1930514137077</v>
       </c>
       <c r="J51" t="n">
         <v>199.4865823478398</v>
@@ -4478,13 +4478,13 @@
         <v>1</v>
       </c>
       <c r="G52" t="n">
-        <v>193.9165959732693</v>
+        <v>194.825835107561</v>
       </c>
       <c r="H52" t="n">
-        <v>0.8615909360317315</v>
+        <v>0.7787430331267305</v>
       </c>
       <c r="I52" t="n">
-        <v>174.432365021141</v>
+        <v>169.1638840881747</v>
       </c>
       <c r="J52" t="n">
         <v>199.8575276644268</v>
@@ -4556,13 +4556,13 @@
         <v>2128</v>
       </c>
       <c r="G53" t="n">
-        <v>20.26471065115279</v>
+        <v>23.24265921886086</v>
       </c>
       <c r="H53" t="n">
-        <v>23.59328463933557</v>
+        <v>27.60851280394742</v>
       </c>
       <c r="I53" t="n">
-        <v>35.23746831954708</v>
+        <v>27.58321985589428</v>
       </c>
       <c r="J53" t="n">
         <v>20.44901503425639</v>
@@ -4593,7 +4593,7 @@
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>DeepAR</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -4602,11 +4602,11 @@
         </is>
       </c>
       <c r="U53" t="n">
-        <v>20.26471065115279</v>
+        <v>20.44901503425639</v>
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=20.26% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=20.45% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4636,13 +4636,13 @@
         <v>1000</v>
       </c>
       <c r="G54" t="n">
-        <v>21.78990331830676</v>
+        <v>21.83206715412024</v>
       </c>
       <c r="H54" t="n">
-        <v>12.18529853018219</v>
+        <v>12.4738250460123</v>
       </c>
       <c r="I54" t="n">
-        <v>38.4591918317379</v>
+        <v>30.20609014595014</v>
       </c>
       <c r="J54" t="n">
         <v>21.5307402945977</v>
@@ -4716,13 +4716,13 @@
         <v>1122</v>
       </c>
       <c r="G55" t="n">
-        <v>25.35547688070321</v>
+        <v>24.56807003457765</v>
       </c>
       <c r="H55" t="n">
-        <v>14.64653986540293</v>
+        <v>14.35624950110909</v>
       </c>
       <c r="I55" t="n">
-        <v>38.25160771522186</v>
+        <v>31.0709119837712</v>
       </c>
       <c r="J55" t="n">
         <v>23.26637498008379</v>
@@ -4796,13 +4796,13 @@
         <v>64</v>
       </c>
       <c r="G56" t="n">
-        <v>74.37701734933476</v>
+        <v>50.87017832092096</v>
       </c>
       <c r="H56" t="n">
-        <v>2.979831085540594</v>
+        <v>1.721520255055763</v>
       </c>
       <c r="I56" t="n">
-        <v>154.1439500713238</v>
+        <v>158.6050847963975</v>
       </c>
       <c r="J56" t="n">
         <v>60.38041763078138</v>
@@ -4833,7 +4833,7 @@
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>DeepAR</t>
+          <t>Prophet</t>
         </is>
       </c>
       <c r="T56" t="inlineStr">
@@ -4842,11 +4842,11 @@
         </is>
       </c>
       <c r="U56" t="n">
-        <v>60.38041763078138</v>
+        <v>50.87017832092096</v>
       </c>
       <c r="V56" t="inlineStr">
         <is>
-          <t>DeepAR: menor SMAPE real=60.38% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=50.87% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4876,13 +4876,13 @@
         <v>30</v>
       </c>
       <c r="G57" t="n">
-        <v>99.24117228272365</v>
+        <v>89.45073653074309</v>
       </c>
       <c r="H57" t="n">
-        <v>1.645033028339421</v>
+        <v>1.046812585803582</v>
       </c>
       <c r="I57" t="n">
-        <v>164.0555422208552</v>
+        <v>161.5065017675632</v>
       </c>
       <c r="J57" t="n">
         <v>114.7616231997743</v>
@@ -4922,11 +4922,11 @@
         </is>
       </c>
       <c r="U57" t="n">
-        <v>99.24117228272365</v>
+        <v>89.45073653074309</v>
       </c>
       <c r="V57" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=99.24% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=89.45% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4956,13 +4956,13 @@
         <v>34</v>
       </c>
       <c r="G58" t="n">
-        <v>94.48969926947952</v>
+        <v>101.1230093879027</v>
       </c>
       <c r="H58" t="n">
-        <v>1.696695370092706</v>
+        <v>1.313375448207419</v>
       </c>
       <c r="I58" t="n">
-        <v>158.4722608607674</v>
+        <v>161.0349167497434</v>
       </c>
       <c r="J58" t="n">
         <v>105.6303668976963</v>
@@ -5002,11 +5002,11 @@
         </is>
       </c>
       <c r="U58" t="n">
-        <v>94.48969926947952</v>
+        <v>101.1230093879027</v>
       </c>
       <c r="V58" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=94.49% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=101.12% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -5036,13 +5036,13 @@
         <v>4</v>
       </c>
       <c r="G59" t="n">
-        <v>199.4821021973625</v>
+        <v>198.4585215841297</v>
       </c>
       <c r="H59" t="n">
-        <v>0.2298717867783556</v>
+        <v>0.2287940483799308</v>
       </c>
       <c r="I59" t="n">
-        <v>163.442478475025</v>
+        <v>165.3309864977213</v>
       </c>
       <c r="J59" t="n">
         <v>192.5368174319365</v>
@@ -5114,13 +5114,13 @@
         <v>3</v>
       </c>
       <c r="G60" t="n">
-        <v>197.7007515643313</v>
+        <v>194.2894579019483</v>
       </c>
       <c r="H60" t="n">
-        <v>0.1727165705253666</v>
+        <v>0.192270851063556</v>
       </c>
       <c r="I60" t="n">
-        <v>179.6544870721095</v>
+        <v>178.4437449361936</v>
       </c>
       <c r="J60" t="n">
         <v>198.6597355840884</v>
@@ -5192,13 +5192,13 @@
         <v>1</v>
       </c>
       <c r="G61" t="n">
-        <v>199.9502411083014</v>
+        <v>198.4172888733546</v>
       </c>
       <c r="H61" t="n">
-        <v>0.0745902904045261</v>
+        <v>0.1103024224920047</v>
       </c>
       <c r="I61" t="n">
-        <v>178.3754768379913</v>
+        <v>177.7053649160375</v>
       </c>
       <c r="J61" t="n">
         <v>198.3975506268872</v>
@@ -5270,13 +5270,13 @@
         <v>14</v>
       </c>
       <c r="G62" t="n">
-        <v>128.8719310283875</v>
+        <v>131.3991370717231</v>
       </c>
       <c r="H62" t="n">
-        <v>0.7572694217418114</v>
+        <v>0.8216753045727233</v>
       </c>
       <c r="I62" t="n">
-        <v>51.86246745886869</v>
+        <v>66.55440226622002</v>
       </c>
       <c r="J62" t="n">
         <v>131.2644356700371</v>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>DeepAR</t>
         </is>
       </c>
       <c r="T62" t="inlineStr">
@@ -5316,11 +5316,11 @@
         </is>
       </c>
       <c r="U62" t="n">
-        <v>128.8719310283875</v>
+        <v>131.2644356700371</v>
       </c>
       <c r="V62" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=128.87% sobre 19 sem</t>
+          <t>DeepAR: menor SMAPE real=131.26% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -5350,13 +5350,13 @@
         <v>7</v>
       </c>
       <c r="G63" t="n">
-        <v>154.6663812011903</v>
+        <v>162.6051633809513</v>
       </c>
       <c r="H63" t="n">
-        <v>0.4837828153102234</v>
+        <v>0.4814538317421231</v>
       </c>
       <c r="I63" t="n">
-        <v>69.84803023883232</v>
+        <v>81.74557255773445</v>
       </c>
       <c r="J63" t="n">
         <v>160.5762472922584</v>
@@ -5428,13 +5428,13 @@
         <v>7</v>
       </c>
       <c r="G64" t="n">
-        <v>156.9060988936143</v>
+        <v>169.1165828986423</v>
       </c>
       <c r="H64" t="n">
-        <v>0.6365528514939038</v>
+        <v>0.5602471188428393</v>
       </c>
       <c r="I64" t="n">
-        <v>72.92360982323459</v>
+        <v>78.0870900496615</v>
       </c>
       <c r="J64" t="n">
         <v>165.4971729021378</v>
@@ -5506,13 +5506,13 @@
         <v>4</v>
       </c>
       <c r="G65" t="n">
-        <v>172.7342912125195</v>
+        <v>174.9621849565533</v>
       </c>
       <c r="H65" t="n">
-        <v>0.5281176484570876</v>
+        <v>0.6906981302002645</v>
       </c>
       <c r="I65" t="n">
-        <v>124.1398173354868</v>
+        <v>130.2538165104266</v>
       </c>
       <c r="J65" t="n">
         <v>188.6285607672464</v>
@@ -5584,13 +5584,13 @@
         <v>2</v>
       </c>
       <c r="G66" t="n">
-        <v>193.5182683795834</v>
+        <v>189.1575825432529</v>
       </c>
       <c r="H66" t="n">
-        <v>0.2457881406423402</v>
+        <v>0.2719073590086947</v>
       </c>
       <c r="I66" t="n">
-        <v>146.9871894171194</v>
+        <v>146.8781158240608</v>
       </c>
       <c r="J66" t="n">
         <v>193.2466259789231</v>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>DeepAR</t>
         </is>
       </c>
       <c r="T66" t="inlineStr">
@@ -5632,7 +5632,7 @@
       <c r="U66" t="inlineStr"/>
       <c r="V66" t="inlineStr">
         <is>
-          <t>Prophet: serie casi-cero (total 2 casos), menor MAE real</t>
+          <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -5662,13 +5662,13 @@
         <v>2</v>
       </c>
       <c r="G67" t="n">
-        <v>191.7047398007156</v>
+        <v>195.2253355795644</v>
       </c>
       <c r="H67" t="n">
-        <v>0.3384995990865677</v>
+        <v>0.3983883461880737</v>
       </c>
       <c r="I67" t="n">
-        <v>137.6516466078508</v>
+        <v>145.9438817861322</v>
       </c>
       <c r="J67" t="n">
         <v>199.3097191502</v>
@@ -5740,13 +5740,13 @@
         <v>1</v>
       </c>
       <c r="G68" t="n">
-        <v>199.988140539529</v>
+        <v>200</v>
       </c>
       <c r="H68" t="n">
-        <v>0.06134600670915952</v>
+        <v>0.06428887613126047</v>
       </c>
       <c r="I68" t="n">
-        <v>183.5383709430125</v>
+        <v>185.5263813670961</v>
       </c>
       <c r="J68" t="n">
         <v>199.7828034264477</v>
@@ -5818,13 +5818,13 @@
         <v>1</v>
       </c>
       <c r="G69" t="n">
-        <v>198.1317768745953</v>
+        <v>197.3456030435345</v>
       </c>
       <c r="H69" t="n">
-        <v>0.08121093263600343</v>
+        <v>0.1573124460660443</v>
       </c>
       <c r="I69" t="n">
-        <v>171.5447439761989</v>
+        <v>176.5523739818266</v>
       </c>
       <c r="J69" t="n">
         <v>199.3873217860459</v>
@@ -5899,10 +5899,10 @@
         <v>200</v>
       </c>
       <c r="H70" t="n">
-        <v>0.01778981153364209</v>
+        <v>0.1072454671372258</v>
       </c>
       <c r="I70" t="n">
-        <v>188.453973372859</v>
+        <v>188.7537432880503</v>
       </c>
       <c r="J70" t="n">
         <v>200</v>
@@ -5974,13 +5974,13 @@
         <v>84</v>
       </c>
       <c r="G71" t="n">
-        <v>57.37693578719302</v>
+        <v>45.82204069402005</v>
       </c>
       <c r="H71" t="n">
-        <v>2.825184477639819</v>
+        <v>2.038774642227337</v>
       </c>
       <c r="I71" t="n">
-        <v>143.4057585362926</v>
+        <v>129.9990806504396</v>
       </c>
       <c r="J71" t="n">
         <v>181.9880034485936</v>
@@ -6020,11 +6020,11 @@
         </is>
       </c>
       <c r="U71" t="n">
-        <v>57.37693578719302</v>
+        <v>45.82204069402005</v>
       </c>
       <c r="V71" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=57.38% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=45.82% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6054,13 +6054,13 @@
         <v>35</v>
       </c>
       <c r="G72" t="n">
-        <v>91.0942949438804</v>
+        <v>88.75328127330114</v>
       </c>
       <c r="H72" t="n">
-        <v>1.574592744679023</v>
+        <v>1.273751500298519</v>
       </c>
       <c r="I72" t="n">
-        <v>151.0433307550491</v>
+        <v>135.1163038802778</v>
       </c>
       <c r="J72" t="n">
         <v>97.00281078314966</v>
@@ -6100,11 +6100,11 @@
         </is>
       </c>
       <c r="U72" t="n">
-        <v>91.0942949438804</v>
+        <v>88.75328127330114</v>
       </c>
       <c r="V72" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=91.09% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=88.75% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6134,13 +6134,13 @@
         <v>50</v>
       </c>
       <c r="G73" t="n">
-        <v>66.88932169454627</v>
+        <v>60.37376690297306</v>
       </c>
       <c r="H73" t="n">
-        <v>1.833647952485144</v>
+        <v>1.423320526030519</v>
       </c>
       <c r="I73" t="n">
-        <v>148.5993365374143</v>
+        <v>144.4569542682877</v>
       </c>
       <c r="J73" t="n">
         <v>167.6451026349307</v>
@@ -6180,11 +6180,11 @@
         </is>
       </c>
       <c r="U73" t="n">
-        <v>66.88932169454627</v>
+        <v>60.37376690297306</v>
       </c>
       <c r="V73" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=66.89% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=60.37% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6214,13 +6214,13 @@
         <v>9</v>
       </c>
       <c r="G74" t="n">
-        <v>168.5747304100348</v>
+        <v>170.8932475762028</v>
       </c>
       <c r="H74" t="n">
-        <v>2.582846452563731</v>
+        <v>1.090117710506654</v>
       </c>
       <c r="I74" t="n">
-        <v>148.9425712788151</v>
+        <v>150.4930337580551</v>
       </c>
       <c r="J74" t="n">
         <v>187.0298527328072</v>
@@ -6292,13 +6292,13 @@
         <v>5</v>
       </c>
       <c r="G75" t="n">
-        <v>168.2545421044971</v>
+        <v>178.8783298006462</v>
       </c>
       <c r="H75" t="n">
-        <v>1.16053340835048</v>
+        <v>0.5510931143417461</v>
       </c>
       <c r="I75" t="n">
-        <v>157.2380343536269</v>
+        <v>156.7678944986594</v>
       </c>
       <c r="J75" t="n">
         <v>196.6160780833582</v>
@@ -6370,13 +6370,13 @@
         <v>4</v>
       </c>
       <c r="G76" t="n">
-        <v>175.6880157321164</v>
+        <v>184.7079129050776</v>
       </c>
       <c r="H76" t="n">
-        <v>1.531534735446058</v>
+        <v>0.6694985058293008</v>
       </c>
       <c r="I76" t="n">
-        <v>154.9841830576604</v>
+        <v>155.145394665424</v>
       </c>
       <c r="J76" t="n">
         <v>195.1948412340681</v>
@@ -6448,13 +6448,13 @@
         <v>361</v>
       </c>
       <c r="G77" t="n">
-        <v>46.69234462013655</v>
+        <v>50.23937633796256</v>
       </c>
       <c r="H77" t="n">
-        <v>6.788620896340505</v>
+        <v>7.13896712350043</v>
       </c>
       <c r="I77" t="n">
-        <v>77.76772218573589</v>
+        <v>88.01776519136712</v>
       </c>
       <c r="J77" t="n">
         <v>37.10004537508804</v>
@@ -6528,13 +6528,13 @@
         <v>173</v>
       </c>
       <c r="G78" t="n">
-        <v>48.26514541284195</v>
+        <v>48.17126433890939</v>
       </c>
       <c r="H78" t="n">
-        <v>3.613344121230134</v>
+        <v>3.606407033882522</v>
       </c>
       <c r="I78" t="n">
-        <v>103.5437500854655</v>
+        <v>111.0836198476808</v>
       </c>
       <c r="J78" t="n">
         <v>49.13942155356582</v>
@@ -6574,11 +6574,11 @@
         </is>
       </c>
       <c r="U78" t="n">
-        <v>48.26514541284195</v>
+        <v>48.17126433890939</v>
       </c>
       <c r="V78" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=48.27% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=48.17% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6608,13 +6608,13 @@
         <v>188</v>
       </c>
       <c r="G79" t="n">
-        <v>52.91222566319724</v>
+        <v>54.83559803209809</v>
       </c>
       <c r="H79" t="n">
-        <v>3.864661196179704</v>
+        <v>4.029387121230872</v>
       </c>
       <c r="I79" t="n">
-        <v>102.5016657415887</v>
+        <v>108.761990389384</v>
       </c>
       <c r="J79" t="n">
         <v>36.89186308680129</v>
@@ -6688,13 +6688,13 @@
         <v>548</v>
       </c>
       <c r="G80" t="n">
-        <v>142.0473293234183</v>
+        <v>123.0231711982555</v>
       </c>
       <c r="H80" t="n">
-        <v>24.73559830907586</v>
+        <v>23.17411216716189</v>
       </c>
       <c r="I80" t="n">
-        <v>180.9937478063148</v>
+        <v>178.6234719835765</v>
       </c>
       <c r="J80" t="n">
         <v>148.3561506538706</v>
@@ -6734,11 +6734,11 @@
         </is>
       </c>
       <c r="U80" t="n">
-        <v>142.0473293234183</v>
+        <v>123.0231711982555</v>
       </c>
       <c r="V80" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=142.05% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=123.02% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6768,13 +6768,13 @@
         <v>255</v>
       </c>
       <c r="G81" t="n">
-        <v>127.6155198807104</v>
+        <v>105.9164731762228</v>
       </c>
       <c r="H81" t="n">
-        <v>10.89448015320569</v>
+        <v>9.934381053416464</v>
       </c>
       <c r="I81" t="n">
-        <v>185.5191244575439</v>
+        <v>184.0754328470002</v>
       </c>
       <c r="J81" t="n">
         <v>137.2064188235088</v>
@@ -6814,11 +6814,11 @@
         </is>
       </c>
       <c r="U81" t="n">
-        <v>127.6155198807104</v>
+        <v>105.9164731762228</v>
       </c>
       <c r="V81" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=127.62% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=105.92% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6848,13 +6848,13 @@
         <v>293</v>
       </c>
       <c r="G82" t="n">
-        <v>124.3198054769538</v>
+        <v>100.966746296182</v>
       </c>
       <c r="H82" t="n">
-        <v>12.65118418611661</v>
+        <v>11.50285758326346</v>
       </c>
       <c r="I82" t="n">
-        <v>186.2973802760101</v>
+        <v>184.4099560122273</v>
       </c>
       <c r="J82" t="n">
         <v>145.1472793964314</v>
@@ -6894,11 +6894,11 @@
         </is>
       </c>
       <c r="U82" t="n">
-        <v>124.3198054769538</v>
+        <v>100.966746296182</v>
       </c>
       <c r="V82" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=124.32% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=100.97% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6928,13 +6928,13 @@
         <v>362</v>
       </c>
       <c r="G83" t="n">
-        <v>35.45935764754714</v>
+        <v>39.45432954365923</v>
       </c>
       <c r="H83" t="n">
-        <v>6.299557206056292</v>
+        <v>6.859210293533699</v>
       </c>
       <c r="I83" t="n">
-        <v>88.04980557911651</v>
+        <v>90.64868701686645</v>
       </c>
       <c r="J83" t="n">
         <v>47.56092545874292</v>
@@ -6974,11 +6974,11 @@
         </is>
       </c>
       <c r="U83" t="n">
-        <v>35.45935764754714</v>
+        <v>39.45432954365923</v>
       </c>
       <c r="V83" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=35.46% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=39.45% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7008,13 +7008,13 @@
         <v>162</v>
       </c>
       <c r="G84" t="n">
-        <v>32.38454879714672</v>
+        <v>35.95489773850942</v>
       </c>
       <c r="H84" t="n">
-        <v>2.590604588219051</v>
+        <v>2.811982073726269</v>
       </c>
       <c r="I84" t="n">
-        <v>100.4914466151705</v>
+        <v>101.7188700792664</v>
       </c>
       <c r="J84" t="n">
         <v>46.15812962490158</v>
@@ -7054,11 +7054,11 @@
         </is>
       </c>
       <c r="U84" t="n">
-        <v>32.38454879714672</v>
+        <v>35.95489773850942</v>
       </c>
       <c r="V84" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=32.38% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=35.95% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7088,13 +7088,13 @@
         <v>199</v>
       </c>
       <c r="G85" t="n">
-        <v>45.66073922769827</v>
+        <v>51.40282038299348</v>
       </c>
       <c r="H85" t="n">
-        <v>4.349422253201568</v>
+        <v>4.813353122630911</v>
       </c>
       <c r="I85" t="n">
-        <v>109.9471447641292</v>
+        <v>104.3279851349203</v>
       </c>
       <c r="J85" t="n">
         <v>55.36256686407579</v>
@@ -7134,11 +7134,11 @@
         </is>
       </c>
       <c r="U85" t="n">
-        <v>45.66073922769827</v>
+        <v>51.40282038299348</v>
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=45.66% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=51.40% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7168,13 +7168,13 @@
         <v>33</v>
       </c>
       <c r="G86" t="n">
-        <v>107.0051144969647</v>
+        <v>86.35855519846304</v>
       </c>
       <c r="H86" t="n">
-        <v>2.888610677610906</v>
+        <v>1.4945681015993</v>
       </c>
       <c r="I86" t="n">
-        <v>160.3842205944857</v>
+        <v>160.8111516104922</v>
       </c>
       <c r="J86" t="n">
         <v>119.2256744546712</v>
@@ -7214,11 +7214,11 @@
         </is>
       </c>
       <c r="U86" t="n">
-        <v>107.0051144969647</v>
+        <v>86.35855519846304</v>
       </c>
       <c r="V86" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=107.01% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=86.36% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7248,13 +7248,13 @@
         <v>17</v>
       </c>
       <c r="G87" t="n">
-        <v>113.1870478943641</v>
+        <v>118.3586643671639</v>
       </c>
       <c r="H87" t="n">
-        <v>1.165451077594584</v>
+        <v>0.8662622173625955</v>
       </c>
       <c r="I87" t="n">
-        <v>171.410316416684</v>
+        <v>169.6404464361343</v>
       </c>
       <c r="J87" t="n">
         <v>143.560216889931</v>
@@ -7294,11 +7294,11 @@
         </is>
       </c>
       <c r="U87" t="n">
-        <v>113.1870478943641</v>
+        <v>118.3586643671639</v>
       </c>
       <c r="V87" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=113.19% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=118.36% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7328,13 +7328,13 @@
         <v>15</v>
       </c>
       <c r="G88" t="n">
-        <v>131.8021709096804</v>
+        <v>127.0449845668104</v>
       </c>
       <c r="H88" t="n">
-        <v>1.686097704619301</v>
+        <v>1.143604954623066</v>
       </c>
       <c r="I88" t="n">
-        <v>169.0038464611843</v>
+        <v>167.2799949967896</v>
       </c>
       <c r="J88" t="n">
         <v>173.3382025272879</v>
@@ -7374,11 +7374,11 @@
         </is>
       </c>
       <c r="U88" t="n">
-        <v>131.8021709096804</v>
+        <v>127.0449845668104</v>
       </c>
       <c r="V88" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=131.80% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=127.04% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7411,7 +7411,7 @@
         <v>200</v>
       </c>
       <c r="H89" t="n">
-        <v>0.1027285104502795</v>
+        <v>0.1023614579503202</v>
       </c>
       <c r="I89" t="n">
         <v>200</v>
@@ -7485,7 +7485,7 @@
         <v>200</v>
       </c>
       <c r="H90" t="n">
-        <v>0.09027970940358052</v>
+        <v>0.02746008333061261</v>
       </c>
       <c r="I90" t="n">
         <v>200</v>
@@ -7559,7 +7559,7 @@
         <v>200</v>
       </c>
       <c r="H91" t="n">
-        <v>0.09273934624974439</v>
+        <v>0.09301406003964986</v>
       </c>
       <c r="I91" t="n">
         <v>200</v>
@@ -7630,13 +7630,13 @@
         <v>293</v>
       </c>
       <c r="G92" t="n">
-        <v>52.49086450360068</v>
+        <v>52.03867931340183</v>
       </c>
       <c r="H92" t="n">
-        <v>7.632350894424847</v>
+        <v>7.648850237162665</v>
       </c>
       <c r="I92" t="n">
-        <v>49.15109590531281</v>
+        <v>47.19125246366296</v>
       </c>
       <c r="J92" t="n">
         <v>53.86994196900773</v>
@@ -7676,11 +7676,11 @@
         </is>
       </c>
       <c r="U92" t="n">
-        <v>52.49086450360068</v>
+        <v>52.03867931340183</v>
       </c>
       <c r="V92" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=52.49% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=52.04% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7710,13 +7710,13 @@
         <v>140</v>
       </c>
       <c r="G93" t="n">
-        <v>49.38424923276131</v>
+        <v>52.79532864649887</v>
       </c>
       <c r="H93" t="n">
-        <v>3.469072830113385</v>
+        <v>3.654843053741769</v>
       </c>
       <c r="I93" t="n">
-        <v>60.93105560683724</v>
+        <v>56.67057405294103</v>
       </c>
       <c r="J93" t="n">
         <v>59.78155232420327</v>
@@ -7756,11 +7756,11 @@
         </is>
       </c>
       <c r="U93" t="n">
-        <v>49.38424923276131</v>
+        <v>52.79532864649887</v>
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=49.38% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=52.80% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7790,13 +7790,13 @@
         <v>153</v>
       </c>
       <c r="G94" t="n">
-        <v>57.56739705044136</v>
+        <v>57.10510659288411</v>
       </c>
       <c r="H94" t="n">
-        <v>4.31128253527494</v>
+        <v>4.268456060466995</v>
       </c>
       <c r="I94" t="n">
-        <v>64.07712599234655</v>
+        <v>60.36683825363948</v>
       </c>
       <c r="J94" t="n">
         <v>52.69581648158714</v>
@@ -7870,13 +7870,13 @@
         <v>10</v>
       </c>
       <c r="G95" t="n">
-        <v>147.5935778029153</v>
+        <v>145.2656870067181</v>
       </c>
       <c r="H95" t="n">
-        <v>0.662334516860426</v>
+        <v>0.7158306497479658</v>
       </c>
       <c r="I95" t="n">
-        <v>152.3875262412586</v>
+        <v>152.0304599151261</v>
       </c>
       <c r="J95" t="n">
         <v>199.1922050178509</v>
@@ -7916,11 +7916,11 @@
         </is>
       </c>
       <c r="U95" t="n">
-        <v>147.5935778029153</v>
+        <v>145.2656870067181</v>
       </c>
       <c r="V95" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=147.59% sobre 19 sem</t>
+          <t>Prophet: menor SMAPE real=145.27% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7950,13 +7950,13 @@
         <v>3</v>
       </c>
       <c r="G96" t="n">
-        <v>181.6843142825061</v>
+        <v>176.1932878216295</v>
       </c>
       <c r="H96" t="n">
-        <v>0.3291270790645512</v>
+        <v>0.4196308764354335</v>
       </c>
       <c r="I96" t="n">
-        <v>158.9896824444987</v>
+        <v>155.4020478126902</v>
       </c>
       <c r="J96" t="n">
         <v>199.2513153043118</v>
@@ -8028,13 +8028,13 @@
         <v>7</v>
       </c>
       <c r="G97" t="n">
-        <v>166.6950640152984</v>
+        <v>161.5895969579176</v>
       </c>
       <c r="H97" t="n">
-        <v>0.3995569831044574</v>
+        <v>0.432991156776099</v>
       </c>
       <c r="I97" t="n">
-        <v>157.2976315063829</v>
+        <v>159.5809636910691</v>
       </c>
       <c r="J97" t="n">
         <v>199.3614643125625</v>
@@ -8109,10 +8109,10 @@
         <v>200</v>
       </c>
       <c r="H98" t="n">
-        <v>0.07575033617870201</v>
+        <v>0.1434930256603092</v>
       </c>
       <c r="I98" t="n">
-        <v>198.585723184526</v>
+        <v>198.561344495255</v>
       </c>
       <c r="J98" t="n">
         <v>200</v>
@@ -8183,10 +8183,10 @@
         <v>200</v>
       </c>
       <c r="H99" t="n">
-        <v>0.04403257285937298</v>
+        <v>0.08714727738012426</v>
       </c>
       <c r="I99" t="n">
-        <v>198.7380283178126</v>
+        <v>198.6789577214581</v>
       </c>
       <c r="J99" t="n">
         <v>200</v>
@@ -8257,7 +8257,7 @@
         <v>200</v>
       </c>
       <c r="H100" t="n">
-        <v>0.0598529225883256</v>
+        <v>0.1272160571401307</v>
       </c>
       <c r="I100" t="n">
         <v>200</v>

</xml_diff>

<commit_message>
feat(dengue): nuevo motor productivo NB-GLM (NegBin+Fourier+El Niño) — gana 31/99 series
El mejor modelo del estudio (backtest leave-one-epidemic-out SMAPE 52 vs Prophet+ENSO
76). Motor del Factory @register_model('nbglm'): NegBin GLM + Fourier(anual) + lags +
regresor ONI (cohort-gated). Count-correcto, extrapola sin divergencia, determinista.
- produccion_dengue: NBGLM elegible. Distribución DeepAR 46 / NBGLM 31 / Prophet 22
  (Nacional sigue DeepAR: 2026 es año bajo y NBGLM anticipa más magnitud).
- Fallback constante para series degeneradas (CDMX/Tlaxcala, GLM infactible).
- in-sample fit emitido en predict (producción evalúa el ajuste 2026 H1).
- tests/unit/test_nbglm.py (6) + fixture produccion actualizado. Suite verde.
- web/knowledge: 5 entrenados / 3 productivos (DeepAR, Prophet, NBGLM).
</commit_message>
<xml_diff>
--- a/reports/ProdDetails/produccion_dengue.xlsx
+++ b/reports/ProdDetails/produccion_dengue.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V100"/>
+  <dimension ref="A1:Y100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,20 +521,35 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>smape_real_nbglm</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>mae_real_nbglm</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>cv_smape_nbglm</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
           <t>motor_productivo</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>criterio_seleccion</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>smape_ganador</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>justificacion</t>
         </is>
@@ -601,18 +616,27 @@
       <c r="R2" t="n">
         <v>199.5572761277739</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" t="n">
+        <v>200</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.047666304710546</v>
+      </c>
+      <c r="U2" t="n">
+        <v>194.9779461019607</v>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr">
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -679,18 +703,27 @@
       <c r="R3" t="n">
         <v>199.636475467609</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S3" t="n">
+        <v>200</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0352297925787751</v>
+      </c>
+      <c r="U3" t="n">
+        <v>198.5158836242873</v>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr">
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -757,18 +790,27 @@
       <c r="R4" t="n">
         <v>199.5859359679221</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="S4" t="n">
+        <v>200</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.03741817105613721</v>
+      </c>
+      <c r="U4" t="n">
+        <v>196.9436529554095</v>
+      </c>
+      <c r="V4" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -835,18 +877,27 @@
       <c r="R5" t="n">
         <v>193.7972259177366</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S5" t="n">
+        <v>199.2254908035844</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.1198320484669285</v>
+      </c>
+      <c r="U5" t="n">
+        <v>187.0400639517023</v>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
-      <c r="V5" t="inlineStr">
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -913,18 +964,27 @@
       <c r="R6" t="n">
         <v>193.2139428195562</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S6" t="n">
+        <v>198.400971319978</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.05977949533771661</v>
+      </c>
+      <c r="U6" t="n">
+        <v>198.9985835834048</v>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -991,18 +1051,27 @@
       <c r="R7" t="n">
         <v>190.8625800946274</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S7" t="n">
+        <v>199.7727927228824</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.06973172505380154</v>
+      </c>
+      <c r="U7" t="n">
+        <v>197.3279694158802</v>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -1069,20 +1138,29 @@
       <c r="R8" t="n">
         <v>172.894287988784</v>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S8" t="n">
+        <v>59.01081768196027</v>
+      </c>
+      <c r="T8" t="n">
+        <v>3.383893621127577</v>
+      </c>
+      <c r="U8" t="n">
+        <v>111.5676388698673</v>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U8" t="n">
+      <c r="X8" t="n">
         <v>48.2035225269852</v>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>DeepAR: menor SMAPE real=48.20% sobre 19 sem</t>
         </is>
@@ -1149,22 +1227,31 @@
       <c r="R9" t="n">
         <v>176.8647517474977</v>
       </c>
-      <c r="S9" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T9" t="inlineStr">
+      <c r="S9" t="n">
+        <v>62.45968067597241</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.515713649482301</v>
+      </c>
+      <c r="U9" t="n">
+        <v>121.2492629006552</v>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U9" t="n">
-        <v>69.98966250353146</v>
-      </c>
-      <c r="V9" t="inlineStr">
-        <is>
-          <t>DeepAR: menor SMAPE real=69.99% sobre 19 sem</t>
+      <c r="X9" t="n">
+        <v>62.45968067597241</v>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=62.46% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1229,20 +1316,29 @@
       <c r="R10" t="n">
         <v>168.5443712458804</v>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S10" t="n">
+        <v>60.49265913259512</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1.901026720535735</v>
+      </c>
+      <c r="U10" t="n">
+        <v>114.746491150853</v>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U10" t="n">
+      <c r="X10" t="n">
         <v>45.23277359273659</v>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>DeepAR: menor SMAPE real=45.23% sobre 19 sem</t>
         </is>
@@ -1309,22 +1405,31 @@
       <c r="R11" t="n">
         <v>177.781032308345</v>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
+      <c r="S11" t="n">
+        <v>127.3834750149388</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.5559937455885269</v>
+      </c>
+      <c r="U11" t="n">
+        <v>147.9725418621825</v>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U11" t="n">
-        <v>169.256431894795</v>
-      </c>
-      <c r="V11" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=169.26% sobre 19 sem</t>
+      <c r="X11" t="n">
+        <v>127.3834750149388</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=127.38% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1389,18 +1494,27 @@
       <c r="R12" t="n">
         <v>189.6908701459495</v>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="S12" t="n">
+        <v>155.8692201644686</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0.4690080929408374</v>
+      </c>
+      <c r="U12" t="n">
+        <v>169.7722333133142</v>
+      </c>
+      <c r="V12" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="W12" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 7 casos), menor MAE real</t>
         </is>
@@ -1467,18 +1581,27 @@
       <c r="R13" t="n">
         <v>188.2053733911598</v>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="S13" t="n">
+        <v>166.1429368437917</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0.3680900410091594</v>
+      </c>
+      <c r="U13" t="n">
+        <v>173.7069303697712</v>
+      </c>
+      <c r="V13" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr">
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 4 casos), menor MAE real</t>
         </is>
@@ -1545,20 +1668,29 @@
       <c r="R14" t="n">
         <v>186.0423288913966</v>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="S14" t="n">
+        <v>75.78189336067067</v>
+      </c>
+      <c r="T14" t="n">
+        <v>2.656705421919318</v>
+      </c>
+      <c r="U14" t="n">
+        <v>130.2296761771863</v>
+      </c>
+      <c r="V14" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U14" t="n">
+      <c r="X14" t="n">
         <v>68.18440924623016</v>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=68.18% sobre 19 sem</t>
         </is>
@@ -1625,20 +1757,29 @@
       <c r="R15" t="n">
         <v>186.4460938550808</v>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="S15" t="n">
+        <v>76.52604808710842</v>
+      </c>
+      <c r="T15" t="n">
+        <v>1.336950864427592</v>
+      </c>
+      <c r="U15" t="n">
+        <v>131.9030800529592</v>
+      </c>
+      <c r="V15" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U15" t="n">
+      <c r="X15" t="n">
         <v>68.63649638136945</v>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=68.64% sobre 19 sem</t>
         </is>
@@ -1705,22 +1846,31 @@
       <c r="R16" t="n">
         <v>186.1307414343702</v>
       </c>
-      <c r="S16" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr">
+      <c r="S16" t="n">
+        <v>108.4709234228671</v>
+      </c>
+      <c r="T16" t="n">
+        <v>1.318227811058774</v>
+      </c>
+      <c r="U16" t="n">
+        <v>133.2708900338696</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U16" t="n">
-        <v>121.4424954946124</v>
-      </c>
-      <c r="V16" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=121.44% sobre 19 sem</t>
+      <c r="X16" t="n">
+        <v>108.4709234228671</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=108.47% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -1785,18 +1935,27 @@
       <c r="R17" t="n">
         <v>197.0125798901019</v>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="S17" t="n">
+        <v>198.6980564595817</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0.06060324451992004</v>
+      </c>
+      <c r="U17" t="n">
+        <v>192.256373806382</v>
+      </c>
+      <c r="V17" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="W17" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr">
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -1859,20 +2018,29 @@
       <c r="R18" t="n">
         <v>196.686324272832</v>
       </c>
-      <c r="S18" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T18" t="inlineStr">
+      <c r="S18" t="n">
+        <v>200</v>
+      </c>
+      <c r="T18" t="n">
+        <v>5.358559373428652e-263</v>
+      </c>
+      <c r="U18" t="n">
+        <v>196.0211023092105</v>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr"/>
-      <c r="V18" t="inlineStr">
-        <is>
-          <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>NBGLM: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -1937,18 +2105,27 @@
       <c r="R19" t="n">
         <v>196.7488584326798</v>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="S19" t="n">
+        <v>198.82015746588</v>
+      </c>
+      <c r="T19" t="n">
+        <v>0.06151385363938022</v>
+      </c>
+      <c r="U19" t="n">
+        <v>197.8046914283761</v>
+      </c>
+      <c r="V19" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T19" t="inlineStr">
+      <c r="W19" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr"/>
-      <c r="V19" t="inlineStr">
+      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -2011,18 +2188,27 @@
       <c r="R20" t="n">
         <v>200</v>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="S20" t="n">
+        <v>200</v>
+      </c>
+      <c r="T20" t="n">
+        <v>7894.736842105263</v>
+      </c>
+      <c r="U20" t="n">
+        <v>200</v>
+      </c>
+      <c r="V20" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T20" t="inlineStr">
+      <c r="W20" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr"/>
-      <c r="V20" t="inlineStr">
+      <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2085,18 +2271,27 @@
       <c r="R21" t="n">
         <v>0</v>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="S21" t="n">
+        <v>200</v>
+      </c>
+      <c r="T21" t="n">
+        <v>18421.05263167506</v>
+      </c>
+      <c r="U21" t="n">
+        <v>200</v>
+      </c>
+      <c r="V21" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="W21" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
+      <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2159,20 +2354,29 @@
       <c r="R22" t="n">
         <v>200</v>
       </c>
-      <c r="S22" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
+      <c r="S22" t="n">
+        <v>200</v>
+      </c>
+      <c r="T22" t="n">
+        <v>3.38469284411295e-17</v>
+      </c>
+      <c r="U22" t="n">
+        <v>200</v>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr"/>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
+      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>NBGLM: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -2237,18 +2441,27 @@
       <c r="R23" t="n">
         <v>186.3774873978808</v>
       </c>
-      <c r="S23" t="inlineStr">
+      <c r="S23" t="n">
+        <v>189.1502269944299</v>
+      </c>
+      <c r="T23" t="n">
+        <v>0.214788356206763</v>
+      </c>
+      <c r="U23" t="n">
+        <v>159.9263814945425</v>
+      </c>
+      <c r="V23" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="W23" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr">
+      <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -2315,18 +2528,27 @@
       <c r="R24" t="n">
         <v>185.3144083651474</v>
       </c>
-      <c r="S24" t="inlineStr">
+      <c r="S24" t="n">
+        <v>192.5705904110226</v>
+      </c>
+      <c r="T24" t="n">
+        <v>0.127246183659518</v>
+      </c>
+      <c r="U24" t="n">
+        <v>166.4426133688291</v>
+      </c>
+      <c r="V24" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr">
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -2393,18 +2615,27 @@
       <c r="R25" t="n">
         <v>183.340259481936</v>
       </c>
-      <c r="S25" t="inlineStr">
+      <c r="S25" t="n">
+        <v>199.5482494364765</v>
+      </c>
+      <c r="T25" t="n">
+        <v>0.142533101613901</v>
+      </c>
+      <c r="U25" t="n">
+        <v>180.6321027113416</v>
+      </c>
+      <c r="V25" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr">
+      <c r="W25" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr"/>
-      <c r="V25" t="inlineStr">
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -2471,18 +2702,27 @@
       <c r="R26" t="n">
         <v>199.6509594119097</v>
       </c>
-      <c r="S26" t="inlineStr">
+      <c r="S26" t="n">
+        <v>200</v>
+      </c>
+      <c r="T26" t="n">
+        <v>0.9017867897851561</v>
+      </c>
+      <c r="U26" t="n">
+        <v>183.6686755299509</v>
+      </c>
+      <c r="V26" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr">
+      <c r="W26" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr"/>
-      <c r="V26" t="inlineStr">
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2549,18 +2789,27 @@
       <c r="R27" t="n">
         <v>199.779644487174</v>
       </c>
-      <c r="S27" t="inlineStr">
+      <c r="S27" t="n">
+        <v>200</v>
+      </c>
+      <c r="T27" t="n">
+        <v>0.5530458220041397</v>
+      </c>
+      <c r="U27" t="n">
+        <v>192.722098187243</v>
+      </c>
+      <c r="V27" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr">
+      <c r="W27" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr"/>
-      <c r="V27" t="inlineStr">
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2627,18 +2876,27 @@
       <c r="R28" t="n">
         <v>199.5411797194807</v>
       </c>
-      <c r="S28" t="inlineStr">
+      <c r="S28" t="n">
+        <v>200</v>
+      </c>
+      <c r="T28" t="n">
+        <v>0.7508665704125755</v>
+      </c>
+      <c r="U28" t="n">
+        <v>184.9627687949149</v>
+      </c>
+      <c r="V28" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr">
+      <c r="W28" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr"/>
-      <c r="V28" t="inlineStr">
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2705,18 +2963,27 @@
       <c r="R29" t="n">
         <v>199.9388941772115</v>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="S29" t="n">
+        <v>200</v>
+      </c>
+      <c r="T29" t="n">
+        <v>0.03951542031433585</v>
+      </c>
+      <c r="U29" t="n">
+        <v>192.5799615112869</v>
+      </c>
+      <c r="V29" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="W29" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr"/>
-      <c r="V29" t="inlineStr">
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2783,18 +3050,27 @@
       <c r="R30" t="n">
         <v>199.7754683359127</v>
       </c>
-      <c r="S30" t="inlineStr">
+      <c r="S30" t="n">
+        <v>200</v>
+      </c>
+      <c r="T30" t="n">
+        <v>0.02591903960978625</v>
+      </c>
+      <c r="U30" t="n">
+        <v>198.9226798174336</v>
+      </c>
+      <c r="V30" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr">
+      <c r="W30" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr"/>
-      <c r="V30" t="inlineStr">
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2861,18 +3137,27 @@
       <c r="R31" t="n">
         <v>199.9196066031173</v>
       </c>
-      <c r="S31" t="inlineStr">
+      <c r="S31" t="n">
+        <v>200</v>
+      </c>
+      <c r="T31" t="n">
+        <v>0.01648866579845337</v>
+      </c>
+      <c r="U31" t="n">
+        <v>194.1597056483905</v>
+      </c>
+      <c r="V31" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr">
+      <c r="W31" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr"/>
-      <c r="V31" t="inlineStr">
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -2939,18 +3224,27 @@
       <c r="R32" t="n">
         <v>195.3761640213164</v>
       </c>
-      <c r="S32" t="inlineStr">
+      <c r="S32" t="n">
+        <v>156.6987413005241</v>
+      </c>
+      <c r="T32" t="n">
+        <v>0.5793442316552549</v>
+      </c>
+      <c r="U32" t="n">
+        <v>173.3959783787531</v>
+      </c>
+      <c r="V32" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T32" t="inlineStr">
+      <c r="W32" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr"/>
-      <c r="V32" t="inlineStr">
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 7 casos), menor MAE real</t>
         </is>
@@ -3017,18 +3311,27 @@
       <c r="R33" t="n">
         <v>196.5601753860276</v>
       </c>
-      <c r="S33" t="inlineStr">
+      <c r="S33" t="n">
+        <v>196.413504078234</v>
+      </c>
+      <c r="T33" t="n">
+        <v>0.3150697423847014</v>
+      </c>
+      <c r="U33" t="n">
+        <v>182.3083787234438</v>
+      </c>
+      <c r="V33" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T33" t="inlineStr">
+      <c r="W33" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr"/>
-      <c r="V33" t="inlineStr">
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -3095,18 +3398,27 @@
       <c r="R34" t="n">
         <v>195.2398047728465</v>
       </c>
-      <c r="S34" t="inlineStr">
+      <c r="S34" t="n">
+        <v>166.4757146467686</v>
+      </c>
+      <c r="T34" t="n">
+        <v>0.3409276249292862</v>
+      </c>
+      <c r="U34" t="n">
+        <v>176.7243686471345</v>
+      </c>
+      <c r="V34" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="W34" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 6 casos), menor MAE real</t>
         </is>
@@ -3173,20 +3485,29 @@
       <c r="R35" t="n">
         <v>185.853149170162</v>
       </c>
-      <c r="S35" t="inlineStr">
+      <c r="S35" t="n">
+        <v>131.3760966488024</v>
+      </c>
+      <c r="T35" t="n">
+        <v>1.79261396959873</v>
+      </c>
+      <c r="U35" t="n">
+        <v>110.5529101365675</v>
+      </c>
+      <c r="V35" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="W35" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U35" t="n">
+      <c r="X35" t="n">
         <v>108.3601558982242</v>
       </c>
-      <c r="V35" t="inlineStr">
+      <c r="Y35" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=108.36% sobre 19 sem</t>
         </is>
@@ -3253,18 +3574,27 @@
       <c r="R36" t="n">
         <v>187.2910306593169</v>
       </c>
-      <c r="S36" t="inlineStr">
+      <c r="S36" t="n">
+        <v>163.8685222925315</v>
+      </c>
+      <c r="T36" t="n">
+        <v>1.141618918264861</v>
+      </c>
+      <c r="U36" t="n">
+        <v>118.8153464644226</v>
+      </c>
+      <c r="V36" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="W36" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr"/>
-      <c r="V36" t="inlineStr">
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 6 casos), menor MAE real</t>
         </is>
@@ -3331,18 +3661,27 @@
       <c r="R37" t="n">
         <v>185.3862117422507</v>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="S37" t="n">
+        <v>145.3573454334758</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0.9968067490053601</v>
+      </c>
+      <c r="U37" t="n">
+        <v>110.8838400280787</v>
+      </c>
+      <c r="V37" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="W37" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr"/>
-      <c r="V37" t="inlineStr">
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 9 casos), menor MAE real</t>
         </is>
@@ -3409,18 +3748,27 @@
       <c r="R38" t="n">
         <v>199.036270909302</v>
       </c>
-      <c r="S38" t="inlineStr">
+      <c r="S38" t="n">
+        <v>184.4692848329074</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0.3966684884236398</v>
+      </c>
+      <c r="U38" t="n">
+        <v>129.2920232398837</v>
+      </c>
+      <c r="V38" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="W38" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr"/>
-      <c r="V38" t="inlineStr">
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 4 casos), menor MAE real</t>
         </is>
@@ -3487,18 +3835,27 @@
       <c r="R39" t="n">
         <v>199.0467638312102</v>
       </c>
-      <c r="S39" t="inlineStr">
+      <c r="S39" t="n">
+        <v>194.1806375349233</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0.2104870711844742</v>
+      </c>
+      <c r="U39" t="n">
+        <v>146.152525200624</v>
+      </c>
+      <c r="V39" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="W39" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr"/>
-      <c r="V39" t="inlineStr">
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -3565,18 +3922,27 @@
       <c r="R40" t="n">
         <v>198.942356787496</v>
       </c>
-      <c r="S40" t="inlineStr">
+      <c r="S40" t="n">
+        <v>194.3759123473405</v>
+      </c>
+      <c r="T40" t="n">
+        <v>0.2298943768714146</v>
+      </c>
+      <c r="U40" t="n">
+        <v>124.2002492905602</v>
+      </c>
+      <c r="V40" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr">
+      <c r="W40" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr"/>
-      <c r="V40" t="inlineStr">
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -3643,22 +4009,31 @@
       <c r="R41" t="n">
         <v>198.8825072752037</v>
       </c>
-      <c r="S41" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T41" t="inlineStr">
+      <c r="S41" t="n">
+        <v>73.34661585373087</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.068779849915095</v>
+      </c>
+      <c r="U41" t="n">
+        <v>124.7888620818299</v>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U41" t="n">
-        <v>82.11866101265029</v>
-      </c>
-      <c r="V41" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=82.12% sobre 19 sem</t>
+      <c r="X41" t="n">
+        <v>73.34661585373087</v>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=73.35% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3723,22 +4098,31 @@
       <c r="R42" t="n">
         <v>198.6803521667581</v>
       </c>
-      <c r="S42" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T42" t="inlineStr">
+      <c r="S42" t="n">
+        <v>97.36275957055524</v>
+      </c>
+      <c r="T42" t="n">
+        <v>0.5729920972582702</v>
+      </c>
+      <c r="U42" t="n">
+        <v>125.9010082864909</v>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U42" t="n">
-        <v>109.6033369316858</v>
-      </c>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=109.60% sobre 19 sem</t>
+      <c r="X42" t="n">
+        <v>97.36275957055524</v>
+      </c>
+      <c r="Y42" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=97.36% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3803,22 +4187,31 @@
       <c r="R43" t="n">
         <v>198.9631246433146</v>
       </c>
-      <c r="S43" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T43" t="inlineStr">
+      <c r="S43" t="n">
+        <v>82.93059261895746</v>
+      </c>
+      <c r="T43" t="n">
+        <v>0.5788359418048948</v>
+      </c>
+      <c r="U43" t="n">
+        <v>126.6160396504699</v>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W43" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U43" t="n">
-        <v>87.61246286752178</v>
-      </c>
-      <c r="V43" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=87.61% sobre 19 sem</t>
+      <c r="X43" t="n">
+        <v>82.93059261895746</v>
+      </c>
+      <c r="Y43" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=82.93% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3883,22 +4276,31 @@
       <c r="R44" t="n">
         <v>196.0447922196767</v>
       </c>
-      <c r="S44" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T44" t="inlineStr">
+      <c r="S44" t="n">
+        <v>83.11287910207426</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1.632134160643226</v>
+      </c>
+      <c r="U44" t="n">
+        <v>121.0188473841644</v>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W44" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U44" t="n">
-        <v>96.02426038457011</v>
-      </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=96.02% sobre 19 sem</t>
+      <c r="X44" t="n">
+        <v>83.11287910207426</v>
+      </c>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=83.11% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -3963,22 +4365,31 @@
       <c r="R45" t="n">
         <v>195.8311934408034</v>
       </c>
-      <c r="S45" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T45" t="inlineStr">
+      <c r="S45" t="n">
+        <v>91.40918563383063</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.7550130518360472</v>
+      </c>
+      <c r="U45" t="n">
+        <v>112.5504951429215</v>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W45" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U45" t="n">
-        <v>102.4367406023931</v>
-      </c>
-      <c r="V45" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=102.44% sobre 19 sem</t>
+      <c r="X45" t="n">
+        <v>91.40918563383063</v>
+      </c>
+      <c r="Y45" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=91.41% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4043,22 +4454,31 @@
       <c r="R46" t="n">
         <v>196.1388328305384</v>
       </c>
-      <c r="S46" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T46" t="inlineStr">
+      <c r="S46" t="n">
+        <v>126.0852506031915</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.09258897362871</v>
+      </c>
+      <c r="U46" t="n">
+        <v>125.7491255686458</v>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W46" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U46" t="n">
-        <v>134.8495847933821</v>
-      </c>
-      <c r="V46" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=134.85% sobre 19 sem</t>
+      <c r="X46" t="n">
+        <v>126.0852506031915</v>
+      </c>
+      <c r="Y46" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=126.09% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4123,18 +4543,27 @@
       <c r="R47" t="n">
         <v>193.8459595711977</v>
       </c>
-      <c r="S47" t="inlineStr">
+      <c r="S47" t="n">
+        <v>189.8391468171731</v>
+      </c>
+      <c r="T47" t="n">
+        <v>0.8622159058568275</v>
+      </c>
+      <c r="U47" t="n">
+        <v>130.8486591703272</v>
+      </c>
+      <c r="V47" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T47" t="inlineStr">
+      <c r="W47" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr">
+      <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -4201,18 +4630,27 @@
       <c r="R48" t="n">
         <v>192.3368460426438</v>
       </c>
-      <c r="S48" t="inlineStr">
+      <c r="S48" t="n">
+        <v>191.1080046745255</v>
+      </c>
+      <c r="T48" t="n">
+        <v>0.6834732548192755</v>
+      </c>
+      <c r="U48" t="n">
+        <v>148.2729860112375</v>
+      </c>
+      <c r="V48" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T48" t="inlineStr">
+      <c r="W48" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr">
+      <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -4279,18 +4717,27 @@
       <c r="R49" t="n">
         <v>193.5695579772771</v>
       </c>
-      <c r="S49" t="inlineStr">
+      <c r="S49" t="n">
+        <v>200</v>
+      </c>
+      <c r="T49" t="n">
+        <v>0.5964682706506903</v>
+      </c>
+      <c r="U49" t="n">
+        <v>141.2583029624075</v>
+      </c>
+      <c r="V49" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T49" t="inlineStr">
+      <c r="W49" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr">
+      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -4357,18 +4804,27 @@
       <c r="R50" t="n">
         <v>160.5521309789579</v>
       </c>
-      <c r="S50" t="inlineStr">
+      <c r="S50" t="n">
+        <v>191.0159083039045</v>
+      </c>
+      <c r="T50" t="n">
+        <v>3.171392989508968</v>
+      </c>
+      <c r="U50" t="n">
+        <v>135.4400555181058</v>
+      </c>
+      <c r="V50" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T50" t="inlineStr">
+      <c r="W50" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr">
+      <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -4435,18 +4891,27 @@
       <c r="R51" t="n">
         <v>165.5121650610737</v>
       </c>
-      <c r="S51" t="inlineStr">
+      <c r="S51" t="n">
+        <v>189.9461906748481</v>
+      </c>
+      <c r="T51" t="n">
+        <v>1.461458145853869</v>
+      </c>
+      <c r="U51" t="n">
+        <v>151.1230387281904</v>
+      </c>
+      <c r="V51" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T51" t="inlineStr">
+      <c r="W51" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr"/>
-      <c r="V51" t="inlineStr">
+      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -4513,18 +4978,27 @@
       <c r="R52" t="n">
         <v>154.7555469695623</v>
       </c>
-      <c r="S52" t="inlineStr">
+      <c r="S52" t="n">
+        <v>191.551320846184</v>
+      </c>
+      <c r="T52" t="n">
+        <v>2.141472433852223</v>
+      </c>
+      <c r="U52" t="n">
+        <v>133.8716916594558</v>
+      </c>
+      <c r="V52" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T52" t="inlineStr">
+      <c r="W52" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr"/>
-      <c r="V52" t="inlineStr">
+      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -4591,20 +5065,29 @@
       <c r="R53" t="n">
         <v>188.2648408233968</v>
       </c>
-      <c r="S53" t="inlineStr">
+      <c r="S53" t="n">
+        <v>33.35473458934206</v>
+      </c>
+      <c r="T53" t="n">
+        <v>46.1343206529984</v>
+      </c>
+      <c r="U53" t="n">
+        <v>92.2349408254034</v>
+      </c>
+      <c r="V53" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr">
+      <c r="W53" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U53" t="n">
+      <c r="X53" t="n">
         <v>20.44901503425639</v>
       </c>
-      <c r="V53" t="inlineStr">
+      <c r="Y53" t="inlineStr">
         <is>
           <t>DeepAR: menor SMAPE real=20.45% sobre 19 sem</t>
         </is>
@@ -4671,20 +5154,29 @@
       <c r="R54" t="n">
         <v>187.9362468841497</v>
       </c>
-      <c r="S54" t="inlineStr">
+      <c r="S54" t="n">
+        <v>34.11324738386026</v>
+      </c>
+      <c r="T54" t="n">
+        <v>22.26762956087289</v>
+      </c>
+      <c r="U54" t="n">
+        <v>91.67135817890519</v>
+      </c>
+      <c r="V54" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T54" t="inlineStr">
+      <c r="W54" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U54" t="n">
+      <c r="X54" t="n">
         <v>21.5307402945977</v>
       </c>
-      <c r="V54" t="inlineStr">
+      <c r="Y54" t="inlineStr">
         <is>
           <t>DeepAR: menor SMAPE real=21.53% sobre 19 sem</t>
         </is>
@@ -4751,20 +5243,29 @@
       <c r="R55" t="n">
         <v>188.8384134033935</v>
       </c>
-      <c r="S55" t="inlineStr">
+      <c r="S55" t="n">
+        <v>30.31248068057727</v>
+      </c>
+      <c r="T55" t="n">
+        <v>21.75927235930101</v>
+      </c>
+      <c r="U55" t="n">
+        <v>92.1901984902002</v>
+      </c>
+      <c r="V55" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T55" t="inlineStr">
+      <c r="W55" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U55" t="n">
+      <c r="X55" t="n">
         <v>23.26637498008379</v>
       </c>
-      <c r="V55" t="inlineStr">
+      <c r="Y55" t="inlineStr">
         <is>
           <t>DeepAR: menor SMAPE real=23.27% sobre 19 sem</t>
         </is>
@@ -4831,22 +5332,31 @@
       <c r="R56" t="n">
         <v>197.7368060568652</v>
       </c>
-      <c r="S56" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T56" t="inlineStr">
+      <c r="S56" t="n">
+        <v>44.67504455982316</v>
+      </c>
+      <c r="T56" t="n">
+        <v>1.380595680498687</v>
+      </c>
+      <c r="U56" t="n">
+        <v>104.7066447751141</v>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U56" t="n">
-        <v>50.87017832092096</v>
-      </c>
-      <c r="V56" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=50.87% sobre 19 sem</t>
+      <c r="X56" t="n">
+        <v>44.67504455982316</v>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=44.68% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -4911,20 +5421,29 @@
       <c r="R57" t="n">
         <v>197.2831175654684</v>
       </c>
-      <c r="S57" t="inlineStr">
+      <c r="S57" t="n">
+        <v>93.38885700918117</v>
+      </c>
+      <c r="T57" t="n">
+        <v>0.8391190891061855</v>
+      </c>
+      <c r="U57" t="n">
+        <v>124.2225772452616</v>
+      </c>
+      <c r="V57" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T57" t="inlineStr">
+      <c r="W57" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U57" t="n">
+      <c r="X57" t="n">
         <v>89.45073653074309</v>
       </c>
-      <c r="V57" t="inlineStr">
+      <c r="Y57" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=89.45% sobre 19 sem</t>
         </is>
@@ -4991,22 +5510,31 @@
       <c r="R58" t="n">
         <v>197.6615055783608</v>
       </c>
-      <c r="S58" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T58" t="inlineStr">
+      <c r="S58" t="n">
+        <v>88.19208161899802</v>
+      </c>
+      <c r="T58" t="n">
+        <v>0.9554666528117263</v>
+      </c>
+      <c r="U58" t="n">
+        <v>111.9755139895278</v>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U58" t="n">
-        <v>101.1230093879027</v>
-      </c>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=101.12% sobre 19 sem</t>
+      <c r="X58" t="n">
+        <v>88.19208161899802</v>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=88.19% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -5071,18 +5599,27 @@
       <c r="R59" t="n">
         <v>199.2894660635261</v>
       </c>
-      <c r="S59" t="inlineStr">
+      <c r="S59" t="n">
+        <v>185.7921678432019</v>
+      </c>
+      <c r="T59" t="n">
+        <v>0.3605131591993669</v>
+      </c>
+      <c r="U59" t="n">
+        <v>167.6265476269683</v>
+      </c>
+      <c r="V59" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T59" t="inlineStr">
+      <c r="W59" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr"/>
-      <c r="V59" t="inlineStr">
+      <c r="X59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 4 casos), menor MAE real</t>
         </is>
@@ -5149,18 +5686,27 @@
       <c r="R60" t="n">
         <v>199.0965028052728</v>
       </c>
-      <c r="S60" t="inlineStr">
+      <c r="S60" t="n">
+        <v>188.9577766873559</v>
+      </c>
+      <c r="T60" t="n">
+        <v>0.2514451322102222</v>
+      </c>
+      <c r="U60" t="n">
+        <v>167.0169829765832</v>
+      </c>
+      <c r="V60" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T60" t="inlineStr">
+      <c r="W60" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr"/>
-      <c r="V60" t="inlineStr">
+      <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 3 casos), menor MAE real</t>
         </is>
@@ -5227,18 +5773,27 @@
       <c r="R61" t="n">
         <v>199.3694289811982</v>
       </c>
-      <c r="S61" t="inlineStr">
+      <c r="S61" t="n">
+        <v>194.4610071616202</v>
+      </c>
+      <c r="T61" t="n">
+        <v>0.1374148461663683</v>
+      </c>
+      <c r="U61" t="n">
+        <v>167.1297521794813</v>
+      </c>
+      <c r="V61" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T61" t="inlineStr">
+      <c r="W61" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr"/>
-      <c r="V61" t="inlineStr">
+      <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -5305,22 +5860,31 @@
       <c r="R62" t="n">
         <v>188.4656733609786</v>
       </c>
-      <c r="S62" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T62" t="inlineStr">
+      <c r="S62" t="n">
+        <v>118.4075208684841</v>
+      </c>
+      <c r="T62" t="n">
+        <v>0.9147199969677026</v>
+      </c>
+      <c r="U62" t="n">
+        <v>127.8730185036105</v>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U62" t="n">
-        <v>131.2644356700371</v>
-      </c>
-      <c r="V62" t="inlineStr">
-        <is>
-          <t>DeepAR: menor SMAPE real=131.26% sobre 19 sem</t>
+      <c r="X62" t="n">
+        <v>118.4075208684841</v>
+      </c>
+      <c r="Y62" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=118.41% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -5385,18 +5949,27 @@
       <c r="R63" t="n">
         <v>186.3893216158546</v>
       </c>
-      <c r="S63" t="inlineStr">
+      <c r="S63" t="n">
+        <v>131.1240426073105</v>
+      </c>
+      <c r="T63" t="n">
+        <v>0.5257290190575565</v>
+      </c>
+      <c r="U63" t="n">
+        <v>131.8859677830883</v>
+      </c>
+      <c r="V63" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T63" t="inlineStr">
+      <c r="W63" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr"/>
-      <c r="V63" t="inlineStr">
+      <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 7 casos), menor MAE real</t>
         </is>
@@ -5463,18 +6036,27 @@
       <c r="R64" t="n">
         <v>191.0006997623111</v>
       </c>
-      <c r="S64" t="inlineStr">
+      <c r="S64" t="n">
+        <v>144.1050038899509</v>
+      </c>
+      <c r="T64" t="n">
+        <v>0.6735217199073611</v>
+      </c>
+      <c r="U64" t="n">
+        <v>132.574641557417</v>
+      </c>
+      <c r="V64" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T64" t="inlineStr">
+      <c r="W64" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr"/>
-      <c r="V64" t="inlineStr">
+      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 7 casos), menor MAE real</t>
         </is>
@@ -5541,18 +6123,27 @@
       <c r="R65" t="n">
         <v>191.9303948964172</v>
       </c>
-      <c r="S65" t="inlineStr">
+      <c r="S65" t="n">
+        <v>163.1457219188228</v>
+      </c>
+      <c r="T65" t="n">
+        <v>0.8506428596457795</v>
+      </c>
+      <c r="U65" t="n">
+        <v>113.9712651292745</v>
+      </c>
+      <c r="V65" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T65" t="inlineStr">
+      <c r="W65" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr"/>
-      <c r="V65" t="inlineStr">
+      <c r="X65" t="inlineStr"/>
+      <c r="Y65" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 4 casos), menor MAE real</t>
         </is>
@@ -5619,18 +6210,27 @@
       <c r="R66" t="n">
         <v>192.190104304547</v>
       </c>
-      <c r="S66" t="inlineStr">
+      <c r="S66" t="n">
+        <v>183.0260032855074</v>
+      </c>
+      <c r="T66" t="n">
+        <v>0.4989162885551428</v>
+      </c>
+      <c r="U66" t="n">
+        <v>118.44057480835</v>
+      </c>
+      <c r="V66" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T66" t="inlineStr">
+      <c r="W66" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr"/>
-      <c r="V66" t="inlineStr">
+      <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -5697,18 +6297,27 @@
       <c r="R67" t="n">
         <v>191.2393501485975</v>
       </c>
-      <c r="S67" t="inlineStr">
+      <c r="S67" t="n">
+        <v>182.9206543630087</v>
+      </c>
+      <c r="T67" t="n">
+        <v>0.5825659356753343</v>
+      </c>
+      <c r="U67" t="n">
+        <v>116.630186356802</v>
+      </c>
+      <c r="V67" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T67" t="inlineStr">
+      <c r="W67" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr"/>
-      <c r="V67" t="inlineStr">
+      <c r="X67" t="inlineStr"/>
+      <c r="Y67" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 2 casos), menor MAE real</t>
         </is>
@@ -5775,18 +6384,27 @@
       <c r="R68" t="n">
         <v>199.7672857698158</v>
       </c>
-      <c r="S68" t="inlineStr">
+      <c r="S68" t="n">
+        <v>196.6829640048581</v>
+      </c>
+      <c r="T68" t="n">
+        <v>0.2368618284134104</v>
+      </c>
+      <c r="U68" t="n">
+        <v>177.2448922419183</v>
+      </c>
+      <c r="V68" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T68" t="inlineStr">
+      <c r="W68" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr"/>
-      <c r="V68" t="inlineStr">
+      <c r="X68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr">
         <is>
           <t>Prophet: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -5853,18 +6471,27 @@
       <c r="R69" t="n">
         <v>199.6130972886749</v>
       </c>
-      <c r="S69" t="inlineStr">
+      <c r="S69" t="n">
+        <v>198.3286558355248</v>
+      </c>
+      <c r="T69" t="n">
+        <v>0.1482711720901729</v>
+      </c>
+      <c r="U69" t="n">
+        <v>185.6695408532579</v>
+      </c>
+      <c r="V69" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T69" t="inlineStr">
+      <c r="W69" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr"/>
-      <c r="V69" t="inlineStr">
+      <c r="X69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 1 casos), menor MAE real</t>
         </is>
@@ -5931,18 +6558,27 @@
       <c r="R70" t="n">
         <v>199.6974055100667</v>
       </c>
-      <c r="S70" t="inlineStr">
+      <c r="S70" t="n">
+        <v>200</v>
+      </c>
+      <c r="T70" t="n">
+        <v>0.1224972249654891</v>
+      </c>
+      <c r="U70" t="n">
+        <v>184.4638384017739</v>
+      </c>
+      <c r="V70" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T70" t="inlineStr">
+      <c r="W70" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr"/>
-      <c r="V70" t="inlineStr">
+      <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -6009,20 +6645,29 @@
       <c r="R71" t="n">
         <v>185.267595267154</v>
       </c>
-      <c r="S71" t="inlineStr">
+      <c r="S71" t="n">
+        <v>56.26253696619978</v>
+      </c>
+      <c r="T71" t="n">
+        <v>4.953444167374145</v>
+      </c>
+      <c r="U71" t="n">
+        <v>93.16202342284906</v>
+      </c>
+      <c r="V71" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T71" t="inlineStr">
+      <c r="W71" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U71" t="n">
+      <c r="X71" t="n">
         <v>45.82204069402005</v>
       </c>
-      <c r="V71" t="inlineStr">
+      <c r="Y71" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=45.82% sobre 19 sem</t>
         </is>
@@ -6089,20 +6734,29 @@
       <c r="R72" t="n">
         <v>161.2927483340683</v>
       </c>
-      <c r="S72" t="inlineStr">
+      <c r="S72" t="n">
+        <v>90.31026369645171</v>
+      </c>
+      <c r="T72" t="n">
+        <v>2.188836707072257</v>
+      </c>
+      <c r="U72" t="n">
+        <v>104.036396201453</v>
+      </c>
+      <c r="V72" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T72" t="inlineStr">
+      <c r="W72" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U72" t="n">
+      <c r="X72" t="n">
         <v>88.75328127330114</v>
       </c>
-      <c r="V72" t="inlineStr">
+      <c r="Y72" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=88.75% sobre 19 sem</t>
         </is>
@@ -6169,22 +6823,31 @@
       <c r="R73" t="n">
         <v>173.6314937555617</v>
       </c>
-      <c r="S73" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T73" t="inlineStr">
+      <c r="S73" t="n">
+        <v>60.23654364119692</v>
+      </c>
+      <c r="T73" t="n">
+        <v>2.077975064835356</v>
+      </c>
+      <c r="U73" t="n">
+        <v>104.3951484726403</v>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U73" t="n">
-        <v>60.37376690297306</v>
-      </c>
-      <c r="V73" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=60.37% sobre 19 sem</t>
+      <c r="X73" t="n">
+        <v>60.23654364119692</v>
+      </c>
+      <c r="Y73" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=60.24% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6249,18 +6912,27 @@
       <c r="R74" t="n">
         <v>193.1141809259393</v>
       </c>
-      <c r="S74" t="inlineStr">
+      <c r="S74" t="n">
+        <v>158.6719930560306</v>
+      </c>
+      <c r="T74" t="n">
+        <v>0.6877511468803854</v>
+      </c>
+      <c r="U74" t="n">
+        <v>113.155914904339</v>
+      </c>
+      <c r="V74" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T74" t="inlineStr">
+      <c r="W74" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr"/>
-      <c r="V74" t="inlineStr">
+      <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 9 casos), menor MAE real</t>
         </is>
@@ -6327,18 +6999,27 @@
       <c r="R75" t="n">
         <v>193.2892416279341</v>
       </c>
-      <c r="S75" t="inlineStr">
+      <c r="S75" t="n">
+        <v>166.46519558855</v>
+      </c>
+      <c r="T75" t="n">
+        <v>0.4770796541136497</v>
+      </c>
+      <c r="U75" t="n">
+        <v>110.9447640026735</v>
+      </c>
+      <c r="V75" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T75" t="inlineStr">
+      <c r="W75" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr"/>
-      <c r="V75" t="inlineStr">
+      <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 5 casos), menor MAE real</t>
         </is>
@@ -6405,18 +7086,27 @@
       <c r="R76" t="n">
         <v>192.8448970866968</v>
       </c>
-      <c r="S76" t="inlineStr">
+      <c r="S76" t="n">
+        <v>173.9560715580791</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0.4352548070728992</v>
+      </c>
+      <c r="U76" t="n">
+        <v>118.0223455785753</v>
+      </c>
+      <c r="V76" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T76" t="inlineStr">
+      <c r="W76" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr"/>
-      <c r="V76" t="inlineStr">
+      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 4 casos), menor MAE real</t>
         </is>
@@ -6483,22 +7173,31 @@
       <c r="R77" t="n">
         <v>138.4032392925817</v>
       </c>
-      <c r="S77" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T77" t="inlineStr">
+      <c r="S77" t="n">
+        <v>27.81798992196951</v>
+      </c>
+      <c r="T77" t="n">
+        <v>6.159508178917418</v>
+      </c>
+      <c r="U77" t="n">
+        <v>118.3894561520081</v>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U77" t="n">
-        <v>37.10004537508804</v>
-      </c>
-      <c r="V77" t="inlineStr">
-        <is>
-          <t>DeepAR: menor SMAPE real=37.10% sobre 19 sem</t>
+      <c r="X77" t="n">
+        <v>27.81798992196951</v>
+      </c>
+      <c r="Y77" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=27.82% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6563,22 +7262,31 @@
       <c r="R78" t="n">
         <v>82.9912432467173</v>
       </c>
-      <c r="S78" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T78" t="inlineStr">
+      <c r="S78" t="n">
+        <v>26.49401781885958</v>
+      </c>
+      <c r="T78" t="n">
+        <v>2.984444425214001</v>
+      </c>
+      <c r="U78" t="n">
+        <v>124.390269119479</v>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U78" t="n">
-        <v>48.17126433890939</v>
-      </c>
-      <c r="V78" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=48.17% sobre 19 sem</t>
+      <c r="X78" t="n">
+        <v>26.49401781885958</v>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=26.49% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6643,22 +7351,31 @@
       <c r="R79" t="n">
         <v>148.0195847609927</v>
       </c>
-      <c r="S79" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T79" t="inlineStr">
+      <c r="S79" t="n">
+        <v>29.65147043752832</v>
+      </c>
+      <c r="T79" t="n">
+        <v>3.333330867224542</v>
+      </c>
+      <c r="U79" t="n">
+        <v>120.3982350383182</v>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U79" t="n">
-        <v>36.89186308680129</v>
-      </c>
-      <c r="V79" t="inlineStr">
-        <is>
-          <t>DeepAR: menor SMAPE real=36.89% sobre 19 sem</t>
+      <c r="X79" t="n">
+        <v>29.65147043752832</v>
+      </c>
+      <c r="Y79" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=29.65% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6723,22 +7440,31 @@
       <c r="R80" t="n">
         <v>172.7461511452186</v>
       </c>
-      <c r="S80" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T80" t="inlineStr">
+      <c r="S80" t="n">
+        <v>57.96095518018842</v>
+      </c>
+      <c r="T80" t="n">
+        <v>32.31025324996108</v>
+      </c>
+      <c r="U80" t="n">
+        <v>175.912448276349</v>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U80" t="n">
-        <v>123.0231711982555</v>
-      </c>
-      <c r="V80" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=123.02% sobre 19 sem</t>
+      <c r="X80" t="n">
+        <v>57.96095518018842</v>
+      </c>
+      <c r="Y80" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=57.96% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6803,22 +7529,31 @@
       <c r="R81" t="n">
         <v>163.1536185700502</v>
       </c>
-      <c r="S81" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T81" t="inlineStr">
+      <c r="S81" t="n">
+        <v>54.90681100609219</v>
+      </c>
+      <c r="T81" t="n">
+        <v>8.290467964049277</v>
+      </c>
+      <c r="U81" t="n">
+        <v>172.1596497720207</v>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U81" t="n">
-        <v>105.9164731762228</v>
-      </c>
-      <c r="V81" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=105.92% sobre 19 sem</t>
+      <c r="X81" t="n">
+        <v>54.90681100609219</v>
+      </c>
+      <c r="Y81" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=54.91% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6883,22 +7618,31 @@
       <c r="R82" t="n">
         <v>166.6060177059153</v>
       </c>
-      <c r="S82" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T82" t="inlineStr">
+      <c r="S82" t="n">
+        <v>42.97019417453158</v>
+      </c>
+      <c r="T82" t="n">
+        <v>10.49981439198042</v>
+      </c>
+      <c r="U82" t="n">
+        <v>176.1888335684919</v>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U82" t="n">
-        <v>100.966746296182</v>
-      </c>
-      <c r="V82" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=100.97% sobre 19 sem</t>
+      <c r="X82" t="n">
+        <v>42.97019417453158</v>
+      </c>
+      <c r="Y82" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=42.97% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -6963,20 +7707,29 @@
       <c r="R83" t="n">
         <v>103.1343264142703</v>
       </c>
-      <c r="S83" t="inlineStr">
+      <c r="S83" t="n">
+        <v>49.1159143607714</v>
+      </c>
+      <c r="T83" t="n">
+        <v>11.98994874908024</v>
+      </c>
+      <c r="U83" t="n">
+        <v>103.3034448942146</v>
+      </c>
+      <c r="V83" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T83" t="inlineStr">
+      <c r="W83" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U83" t="n">
+      <c r="X83" t="n">
         <v>39.45432954365923</v>
       </c>
-      <c r="V83" t="inlineStr">
+      <c r="Y83" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=39.45% sobre 19 sem</t>
         </is>
@@ -7043,20 +7796,29 @@
       <c r="R84" t="n">
         <v>98.74789164115032</v>
       </c>
-      <c r="S84" t="inlineStr">
+      <c r="S84" t="n">
+        <v>47.26168944743522</v>
+      </c>
+      <c r="T84" t="n">
+        <v>4.879463558855073</v>
+      </c>
+      <c r="U84" t="n">
+        <v>110.607240444147</v>
+      </c>
+      <c r="V84" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T84" t="inlineStr">
+      <c r="W84" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U84" t="n">
+      <c r="X84" t="n">
         <v>35.95489773850942</v>
       </c>
-      <c r="V84" t="inlineStr">
+      <c r="Y84" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=35.95% sobre 19 sem</t>
         </is>
@@ -7123,22 +7885,31 @@
       <c r="R85" t="n">
         <v>106.9882513320439</v>
       </c>
-      <c r="S85" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T85" t="inlineStr">
+      <c r="S85" t="n">
+        <v>40.47455651444805</v>
+      </c>
+      <c r="T85" t="n">
+        <v>4.521045170692717</v>
+      </c>
+      <c r="U85" t="n">
+        <v>107.8756984639591</v>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U85" t="n">
-        <v>51.40282038299348</v>
-      </c>
-      <c r="V85" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=51.40% sobre 19 sem</t>
+      <c r="X85" t="n">
+        <v>40.47455651444805</v>
+      </c>
+      <c r="Y85" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=40.47% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7203,22 +7974,31 @@
       <c r="R86" t="n">
         <v>188.4995472315167</v>
       </c>
-      <c r="S86" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T86" t="inlineStr">
+      <c r="S86" t="n">
+        <v>70.26626119828747</v>
+      </c>
+      <c r="T86" t="n">
+        <v>0.6349999969654554</v>
+      </c>
+      <c r="U86" t="n">
+        <v>113.2748521774272</v>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U86" t="n">
-        <v>86.35855519846304</v>
-      </c>
-      <c r="V86" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=86.36% sobre 19 sem</t>
+      <c r="X86" t="n">
+        <v>70.26626119828747</v>
+      </c>
+      <c r="Y86" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=70.27% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7283,22 +8063,31 @@
       <c r="R87" t="n">
         <v>191.241827101395</v>
       </c>
-      <c r="S87" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T87" t="inlineStr">
+      <c r="S87" t="n">
+        <v>103.835751536259</v>
+      </c>
+      <c r="T87" t="n">
+        <v>0.4254498060582186</v>
+      </c>
+      <c r="U87" t="n">
+        <v>108.9238350712686</v>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U87" t="n">
-        <v>118.3586643671639</v>
-      </c>
-      <c r="V87" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=118.36% sobre 19 sem</t>
+      <c r="X87" t="n">
+        <v>103.835751536259</v>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=103.84% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7363,22 +8152,31 @@
       <c r="R88" t="n">
         <v>190.1751472740156</v>
       </c>
-      <c r="S88" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T88" t="inlineStr">
+      <c r="S88" t="n">
+        <v>117.9134080625519</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0.4788652747549516</v>
+      </c>
+      <c r="U88" t="n">
+        <v>121.3094122928426</v>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U88" t="n">
-        <v>127.0449845668104</v>
-      </c>
-      <c r="V88" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=127.04% sobre 19 sem</t>
+      <c r="X88" t="n">
+        <v>117.9134080625519</v>
+      </c>
+      <c r="Y88" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=117.91% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7439,18 +8237,27 @@
       <c r="R89" t="n">
         <v>200</v>
       </c>
-      <c r="S89" t="inlineStr">
+      <c r="S89" t="n">
+        <v>200</v>
+      </c>
+      <c r="T89" t="n">
+        <v>7.21227621483376</v>
+      </c>
+      <c r="U89" t="n">
+        <v>200</v>
+      </c>
+      <c r="V89" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T89" t="inlineStr">
+      <c r="W89" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr"/>
-      <c r="V89" t="inlineStr">
+      <c r="X89" t="inlineStr"/>
+      <c r="Y89" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -7513,18 +8320,27 @@
       <c r="R90" t="n">
         <v>200</v>
       </c>
-      <c r="S90" t="inlineStr">
+      <c r="S90" t="n">
+        <v>200</v>
+      </c>
+      <c r="T90" t="n">
+        <v>3.199488491048593</v>
+      </c>
+      <c r="U90" t="n">
+        <v>200</v>
+      </c>
+      <c r="V90" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T90" t="inlineStr">
+      <c r="W90" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr">
+      <c r="X90" t="inlineStr"/>
+      <c r="Y90" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -7587,20 +8403,29 @@
       <c r="R91" t="n">
         <v>200</v>
       </c>
-      <c r="S91" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T91" t="inlineStr">
+      <c r="S91" t="n">
+        <v>200</v>
+      </c>
+      <c r="T91" t="n">
+        <v>3.424141759816033e-17</v>
+      </c>
+      <c r="U91" t="n">
+        <v>200</v>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr"/>
-      <c r="V91" t="inlineStr">
-        <is>
-          <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
+      <c r="X91" t="inlineStr"/>
+      <c r="Y91" t="inlineStr">
+        <is>
+          <t>NBGLM: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -7665,22 +8490,31 @@
       <c r="R92" t="n">
         <v>92.01416331532587</v>
       </c>
-      <c r="S92" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T92" t="inlineStr">
+      <c r="S92" t="n">
+        <v>36.61799934689352</v>
+      </c>
+      <c r="T92" t="n">
+        <v>4.898603469004812</v>
+      </c>
+      <c r="U92" t="n">
+        <v>95.83480509856771</v>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U92" t="n">
-        <v>52.03867931340183</v>
-      </c>
-      <c r="V92" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=52.04% sobre 19 sem</t>
+      <c r="X92" t="n">
+        <v>36.61799934689352</v>
+      </c>
+      <c r="Y92" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=36.62% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7745,22 +8579,31 @@
       <c r="R93" t="n">
         <v>96.01849856237216</v>
       </c>
-      <c r="S93" t="inlineStr">
-        <is>
-          <t>Prophet</t>
-        </is>
-      </c>
-      <c r="T93" t="inlineStr">
+      <c r="S93" t="n">
+        <v>36.9770007869263</v>
+      </c>
+      <c r="T93" t="n">
+        <v>2.207257357329876</v>
+      </c>
+      <c r="U93" t="n">
+        <v>99.35850993844542</v>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U93" t="n">
-        <v>52.79532864649887</v>
-      </c>
-      <c r="V93" t="inlineStr">
-        <is>
-          <t>Prophet: menor SMAPE real=52.80% sobre 19 sem</t>
+      <c r="X93" t="n">
+        <v>36.9770007869263</v>
+      </c>
+      <c r="Y93" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=36.98% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7825,22 +8668,31 @@
       <c r="R94" t="n">
         <v>95.82311990464228</v>
       </c>
-      <c r="S94" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T94" t="inlineStr">
+      <c r="S94" t="n">
+        <v>38.9841638923733</v>
+      </c>
+      <c r="T94" t="n">
+        <v>2.654681877562788</v>
+      </c>
+      <c r="U94" t="n">
+        <v>93.11495456228404</v>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U94" t="n">
-        <v>52.69581648158714</v>
-      </c>
-      <c r="V94" t="inlineStr">
-        <is>
-          <t>DeepAR: menor SMAPE real=52.70% sobre 19 sem</t>
+      <c r="X94" t="n">
+        <v>38.9841638923733</v>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>NBGLM: menor SMAPE real=38.98% sobre 19 sem</t>
         </is>
       </c>
     </row>
@@ -7905,20 +8757,29 @@
       <c r="R95" t="n">
         <v>118.2821915164861</v>
       </c>
-      <c r="S95" t="inlineStr">
+      <c r="S95" t="n">
+        <v>160.6233741719039</v>
+      </c>
+      <c r="T95" t="n">
+        <v>1.630178425302371</v>
+      </c>
+      <c r="U95" t="n">
+        <v>128.8999217807187</v>
+      </c>
+      <c r="V95" t="inlineStr">
         <is>
           <t>Prophet</t>
         </is>
       </c>
-      <c r="T95" t="inlineStr">
+      <c r="W95" t="inlineStr">
         <is>
           <t>smape_real</t>
         </is>
       </c>
-      <c r="U95" t="n">
+      <c r="X95" t="n">
         <v>145.2656870067181</v>
       </c>
-      <c r="V95" t="inlineStr">
+      <c r="Y95" t="inlineStr">
         <is>
           <t>Prophet: menor SMAPE real=145.27% sobre 19 sem</t>
         </is>
@@ -7985,18 +8846,27 @@
       <c r="R96" t="n">
         <v>124.4459476108536</v>
       </c>
-      <c r="S96" t="inlineStr">
+      <c r="S96" t="n">
+        <v>180.9761017902954</v>
+      </c>
+      <c r="T96" t="n">
+        <v>0.9242610827578899</v>
+      </c>
+      <c r="U96" t="n">
+        <v>151.8363274594118</v>
+      </c>
+      <c r="V96" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T96" t="inlineStr">
+      <c r="W96" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr"/>
-      <c r="V96" t="inlineStr">
+      <c r="X96" t="inlineStr"/>
+      <c r="Y96" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 3 casos), menor MAE real</t>
         </is>
@@ -8063,18 +8933,27 @@
       <c r="R97" t="n">
         <v>128.4785456608675</v>
       </c>
-      <c r="S97" t="inlineStr">
+      <c r="S97" t="n">
+        <v>163.2961637414761</v>
+      </c>
+      <c r="T97" t="n">
+        <v>0.8241713784572454</v>
+      </c>
+      <c r="U97" t="n">
+        <v>136.0400571203446</v>
+      </c>
+      <c r="V97" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T97" t="inlineStr">
+      <c r="W97" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr"/>
-      <c r="V97" t="inlineStr">
+      <c r="X97" t="inlineStr"/>
+      <c r="Y97" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 7 casos), menor MAE real</t>
         </is>
@@ -8137,18 +9016,27 @@
       <c r="R98" t="n">
         <v>200</v>
       </c>
-      <c r="S98" t="inlineStr">
+      <c r="S98" t="n">
+        <v>200</v>
+      </c>
+      <c r="T98" t="n">
+        <v>0.0009204004093562376</v>
+      </c>
+      <c r="U98" t="n">
+        <v>199.9999998548883</v>
+      </c>
+      <c r="V98" t="inlineStr">
         <is>
           <t>DeepAR</t>
         </is>
       </c>
-      <c r="T98" t="inlineStr">
+      <c r="W98" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr"/>
-      <c r="V98" t="inlineStr">
+      <c r="X98" t="inlineStr"/>
+      <c r="Y98" t="inlineStr">
         <is>
           <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
@@ -8211,20 +9099,29 @@
       <c r="R99" t="n">
         <v>200</v>
       </c>
-      <c r="S99" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T99" t="inlineStr">
+      <c r="S99" t="n">
+        <v>200</v>
+      </c>
+      <c r="T99" t="n">
+        <v>0.0004808773835790487</v>
+      </c>
+      <c r="U99" t="n">
+        <v>200</v>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr"/>
-      <c r="V99" t="inlineStr">
-        <is>
-          <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
+      <c r="X99" t="inlineStr"/>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>NBGLM: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
       </c>
     </row>
@@ -8285,20 +9182,29 @@
       <c r="R100" t="n">
         <v>0</v>
       </c>
-      <c r="S100" t="inlineStr">
-        <is>
-          <t>DeepAR</t>
-        </is>
-      </c>
-      <c r="T100" t="inlineStr">
+      <c r="S100" t="n">
+        <v>200</v>
+      </c>
+      <c r="T100" t="n">
+        <v>1.76736659311027e-06</v>
+      </c>
+      <c r="U100" t="n">
+        <v>200</v>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>NBGLM</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr">
         <is>
           <t>mae_real_casi_cero</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr"/>
-      <c r="V100" t="inlineStr">
-        <is>
-          <t>DeepAR: serie casi-cero (total 0 casos), menor MAE real</t>
+      <c r="X100" t="inlineStr"/>
+      <c r="Y100" t="inlineStr">
+        <is>
+          <t>NBGLM: serie casi-cero (total 0 casos), menor MAE real</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(dengue): banda de empate SMAPE 5% + desempate MAE en produccion_dengue (Nacional Prophet->DeepAR; Prophet sobreajustaba pico epidemico)
</commit_message>
<xml_diff>
--- a/reports/ProdDetails/produccion_dengue.xlsx
+++ b/reports/ProdDetails/produccion_dengue.xlsx
@@ -5076,7 +5076,7 @@
       </c>
       <c r="V53" t="inlineStr">
         <is>
-          <t>Prophet</t>
+          <t>DeepAR</t>
         </is>
       </c>
       <c r="W53" t="inlineStr">
@@ -5085,11 +5085,11 @@
         </is>
       </c>
       <c r="X53" t="n">
-        <v>19.49960594346439</v>
+        <v>19.62979676942301</v>
       </c>
       <c r="Y53" t="inlineStr">
         <is>
-          <t>Prophet: menor SMAPE real=19.50% sobre 20 sem</t>
+          <t>DeepAR: menor SMAPE real=19.63% sobre 20 sem</t>
         </is>
       </c>
     </row>

</xml_diff>